<commit_message>
Update all.xlsx with latest transaction data revisions
</commit_message>
<xml_diff>
--- a/data/transactions/all.xlsx
+++ b/data/transactions/all.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="23801"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24332"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{416924DF-F880-4F53-89A7-1D98A0CC954C}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D8A7D73-0C59-498C-AF53-91F53B0BB08C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -14,11 +14,22 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A1:$K1578</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8586" uniqueCount="2400">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8586" uniqueCount="2399">
   <si>
     <t>كود الصنف</t>
   </si>
@@ -7104,9 +7115,6 @@
   </si>
   <si>
     <t xml:space="preserve">فاصل زيت </t>
-  </si>
-  <si>
-    <t>19-4-2027</t>
   </si>
   <si>
     <t>6337</t>
@@ -8207,7 +8215,7 @@
     <row r="4" spans="1:15" s="12" customFormat="1" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A4" s="13"/>
       <c r="B4" s="14" t="s">
-        <v>2396</v>
+        <v>2395</v>
       </c>
       <c r="C4" s="15" t="s">
         <v>21</v>
@@ -22786,7 +22794,7 @@
     <row r="409" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A409" s="13"/>
       <c r="B409" s="14" t="s">
-        <v>2397</v>
+        <v>2396</v>
       </c>
       <c r="C409" s="15" t="s">
         <v>21</v>
@@ -25196,7 +25204,7 @@
     <row r="476" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A476" s="13"/>
       <c r="B476" s="14" t="s">
-        <v>2381</v>
+        <v>2380</v>
       </c>
       <c r="C476" s="15" t="s">
         <v>21</v>
@@ -25338,7 +25346,7 @@
     <row r="480" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A480" s="13"/>
       <c r="B480" s="14" t="s">
-        <v>2380</v>
+        <v>2379</v>
       </c>
       <c r="C480" s="15" t="s">
         <v>21</v>
@@ -25408,7 +25416,7 @@
     <row r="482" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A482" s="13"/>
       <c r="B482" s="14" t="s">
-        <v>2379</v>
+        <v>2378</v>
       </c>
       <c r="C482" s="15" t="s">
         <v>21</v>
@@ -25624,7 +25632,7 @@
         <v>2080</v>
       </c>
       <c r="B488" s="14" t="s">
-        <v>2378</v>
+        <v>2377</v>
       </c>
       <c r="C488" s="15" t="s">
         <v>21</v>
@@ -28102,7 +28110,7 @@
     <row r="557" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A557" s="13"/>
       <c r="B557" s="14" t="s">
-        <v>2394</v>
+        <v>2393</v>
       </c>
       <c r="C557" s="15" t="s">
         <v>21</v>
@@ -33245,10 +33253,10 @@
     </row>
     <row r="700" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A700" s="59" t="s">
-        <v>2384</v>
+        <v>2383</v>
       </c>
       <c r="B700" s="14" t="s">
-        <v>2383</v>
+        <v>2382</v>
       </c>
       <c r="C700" s="15" t="s">
         <v>21</v>
@@ -33533,10 +33541,10 @@
     </row>
     <row r="708" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A708" s="59" t="s">
-        <v>2386</v>
+        <v>2385</v>
       </c>
       <c r="B708" s="14" t="s">
-        <v>2385</v>
+        <v>2384</v>
       </c>
       <c r="C708" s="15" t="s">
         <v>21</v>
@@ -34179,10 +34187,10 @@
     </row>
     <row r="726" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A726" s="59" t="s">
-        <v>2386</v>
+        <v>2385</v>
       </c>
       <c r="B726" s="14" t="s">
-        <v>2385</v>
+        <v>2384</v>
       </c>
       <c r="C726" s="15" t="s">
         <v>21</v>
@@ -34215,10 +34223,10 @@
     </row>
     <row r="727" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A727" s="59" t="s">
-        <v>2384</v>
+        <v>2383</v>
       </c>
       <c r="B727" s="14" t="s">
-        <v>2383</v>
+        <v>2382</v>
       </c>
       <c r="C727" s="15" t="s">
         <v>21</v>
@@ -35406,7 +35414,7 @@
         <v>1245</v>
       </c>
       <c r="B760" s="14" t="s">
-        <v>2387</v>
+        <v>2386</v>
       </c>
       <c r="C760" s="15" t="s">
         <v>21</v>
@@ -37380,7 +37388,7 @@
     <row r="815" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A815" s="13"/>
       <c r="B815" s="14" t="s">
-        <v>2388</v>
+        <v>2387</v>
       </c>
       <c r="C815" s="15" t="s">
         <v>21</v>
@@ -38924,7 +38932,7 @@
     <row r="858" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A858" s="13"/>
       <c r="B858" s="14" t="s">
-        <v>2389</v>
+        <v>2388</v>
       </c>
       <c r="C858" s="15" t="s">
         <v>21</v>
@@ -39390,7 +39398,7 @@
     <row r="871" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A871" s="13"/>
       <c r="B871" s="14" t="s">
-        <v>2395</v>
+        <v>2394</v>
       </c>
       <c r="C871" s="15" t="s">
         <v>21</v>
@@ -41334,7 +41342,7 @@
         <v>2277</v>
       </c>
       <c r="B925" s="14" t="s">
-        <v>2377</v>
+        <v>2376</v>
       </c>
       <c r="C925" s="15" t="s">
         <v>21</v>
@@ -42296,7 +42304,7 @@
     <row r="952" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A952" s="13"/>
       <c r="B952" s="14" t="s">
-        <v>2382</v>
+        <v>2381</v>
       </c>
       <c r="C952" s="15" t="s">
         <v>21</v>
@@ -43266,7 +43274,7 @@
     <row r="979" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A979" s="13"/>
       <c r="B979" s="14" t="s">
-        <v>2390</v>
+        <v>2389</v>
       </c>
       <c r="C979" s="15" t="s">
         <v>21</v>
@@ -45672,7 +45680,7 @@
     <row r="1046" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A1046" s="13"/>
       <c r="B1046" s="14" t="s">
-        <v>2398</v>
+        <v>2397</v>
       </c>
       <c r="C1046" s="15" t="s">
         <v>21</v>
@@ -45706,7 +45714,7 @@
     <row r="1047" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A1047" s="13"/>
       <c r="B1047" s="14" t="s">
-        <v>2399</v>
+        <v>2398</v>
       </c>
       <c r="C1047" s="15" t="s">
         <v>21</v>
@@ -47285,7 +47293,7 @@
     </row>
     <row r="1091" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A1091" s="60" t="s">
-        <v>2364</v>
+        <v>2363</v>
       </c>
       <c r="B1091" s="14" t="s">
         <v>2361</v>
@@ -47307,13 +47315,13 @@
         <v>1708</v>
       </c>
       <c r="H1091" s="18" t="s">
-        <v>2362</v>
+        <v>1666</v>
       </c>
       <c r="I1091" s="15" t="s">
         <v>1709</v>
       </c>
       <c r="J1091" s="15" t="s">
-        <v>2363</v>
+        <v>2362</v>
       </c>
       <c r="K1091" s="18">
         <v>46117</v>
@@ -50700,10 +50708,10 @@
     </row>
     <row r="1186" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A1186" s="60" t="s">
-        <v>2376</v>
+        <v>2375</v>
       </c>
       <c r="B1186" s="14" t="s">
-        <v>2375</v>
+        <v>2374</v>
       </c>
       <c r="C1186" s="15" t="s">
         <v>21</v>
@@ -54691,7 +54699,7 @@
     <row r="1297" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A1297" s="13"/>
       <c r="B1297" s="14" t="s">
-        <v>2393</v>
+        <v>2392</v>
       </c>
       <c r="C1297" s="15" t="s">
         <v>21</v>
@@ -56237,7 +56245,7 @@
     <row r="1340" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A1340" s="13"/>
       <c r="B1340" s="62" t="s">
-        <v>2391</v>
+        <v>2390</v>
       </c>
       <c r="C1340" s="15" t="s">
         <v>21</v>
@@ -57566,10 +57574,10 @@
     </row>
     <row r="1377" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A1377" s="60" t="s">
-        <v>2368</v>
+        <v>2367</v>
       </c>
       <c r="B1377" s="14" t="s">
-        <v>2366</v>
+        <v>2365</v>
       </c>
       <c r="C1377" s="15" t="s">
         <v>21</v>
@@ -57602,10 +57610,10 @@
     </row>
     <row r="1378" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A1378" s="60" t="s">
-        <v>2369</v>
+        <v>2368</v>
       </c>
       <c r="B1378" s="14" t="s">
-        <v>2367</v>
+        <v>2366</v>
       </c>
       <c r="C1378" s="15" t="s">
         <v>21</v>
@@ -57674,10 +57682,10 @@
     </row>
     <row r="1380" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A1380" s="60" t="s">
-        <v>2371</v>
+        <v>2370</v>
       </c>
       <c r="B1380" s="14" t="s">
-        <v>2370</v>
+        <v>2369</v>
       </c>
       <c r="C1380" s="15" t="s">
         <v>21</v>
@@ -57746,10 +57754,10 @@
     </row>
     <row r="1382" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A1382" s="60" t="s">
-        <v>2373</v>
+        <v>2372</v>
       </c>
       <c r="B1382" s="14" t="s">
-        <v>2372</v>
+        <v>2371</v>
       </c>
       <c r="C1382" s="15" t="s">
         <v>21</v>
@@ -58538,7 +58546,7 @@
     </row>
     <row r="1404" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A1404" s="60" t="s">
-        <v>2374</v>
+        <v>2373</v>
       </c>
       <c r="B1404" s="14" t="s">
         <v>2103</v>
@@ -59079,7 +59087,7 @@
     <row r="1419" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A1419" s="13"/>
       <c r="B1419" s="14" t="s">
-        <v>2392</v>
+        <v>2391</v>
       </c>
       <c r="C1419" s="15" t="s">
         <v>21</v>
@@ -62365,7 +62373,7 @@
         <v>96</v>
       </c>
       <c r="B1511" s="14" t="s">
-        <v>2365</v>
+        <v>2364</v>
       </c>
       <c r="C1511" s="15" t="s">
         <v>21</v>

</xml_diff>

<commit_message>
Update all.xlsx with the latest transaction data revisions
</commit_message>
<xml_diff>
--- a/data/transactions/all.xlsx
+++ b/data/transactions/all.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24332"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D8A7D73-0C59-498C-AF53-91F53B0BB08C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02CEA2FD-42BA-416C-8F58-88BA7E874C94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7087,24 +7087,12 @@
     <t>فلتر لحام 5/8</t>
   </si>
   <si>
-    <t>بروفيل باب تلاجة PVC موديل A141</t>
-  </si>
-  <si>
     <t>19/4/2026</t>
   </si>
   <si>
     <t>سماريل</t>
   </si>
   <si>
-    <t>بروفيل باب تلاجة PVC موديل A142</t>
-  </si>
-  <si>
-    <t>بروفيل باب تلاجة PVC موديل A143</t>
-  </si>
-  <si>
-    <t>بروفيل باب تلاجة PVC موديل A144</t>
-  </si>
-  <si>
     <t>افرلود 5/8 5</t>
   </si>
   <si>
@@ -7226,6 +7214,18 @@
   </si>
   <si>
     <t>بنطه كبايه 19</t>
+  </si>
+  <si>
+    <t>بروفيل باب ثلاجة PVC موديل A141</t>
+  </si>
+  <si>
+    <t>بروفيل باب ثلاجة PVC موديل A142</t>
+  </si>
+  <si>
+    <t>بروفيل باب ثلاجة PVC موديل A143</t>
+  </si>
+  <si>
+    <t>بروفيل باب ثلاجة PVC موديل A144</t>
   </si>
 </sst>
 </file>
@@ -8215,7 +8215,7 @@
     <row r="4" spans="1:15" s="12" customFormat="1" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A4" s="13"/>
       <c r="B4" s="14" t="s">
-        <v>2395</v>
+        <v>2391</v>
       </c>
       <c r="C4" s="15" t="s">
         <v>21</v>
@@ -22794,7 +22794,7 @@
     <row r="409" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A409" s="13"/>
       <c r="B409" s="14" t="s">
-        <v>2396</v>
+        <v>2392</v>
       </c>
       <c r="C409" s="15" t="s">
         <v>21</v>
@@ -25204,7 +25204,7 @@
     <row r="476" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A476" s="13"/>
       <c r="B476" s="14" t="s">
-        <v>2380</v>
+        <v>2376</v>
       </c>
       <c r="C476" s="15" t="s">
         <v>21</v>
@@ -25346,7 +25346,7 @@
     <row r="480" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A480" s="13"/>
       <c r="B480" s="14" t="s">
-        <v>2379</v>
+        <v>2375</v>
       </c>
       <c r="C480" s="15" t="s">
         <v>21</v>
@@ -25416,7 +25416,7 @@
     <row r="482" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A482" s="13"/>
       <c r="B482" s="14" t="s">
-        <v>2378</v>
+        <v>2374</v>
       </c>
       <c r="C482" s="15" t="s">
         <v>21</v>
@@ -25632,7 +25632,7 @@
         <v>2080</v>
       </c>
       <c r="B488" s="14" t="s">
-        <v>2377</v>
+        <v>2373</v>
       </c>
       <c r="C488" s="15" t="s">
         <v>21</v>
@@ -28110,7 +28110,7 @@
     <row r="557" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A557" s="13"/>
       <c r="B557" s="14" t="s">
-        <v>2393</v>
+        <v>2389</v>
       </c>
       <c r="C557" s="15" t="s">
         <v>21</v>
@@ -33253,10 +33253,10 @@
     </row>
     <row r="700" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A700" s="59" t="s">
-        <v>2383</v>
+        <v>2379</v>
       </c>
       <c r="B700" s="14" t="s">
-        <v>2382</v>
+        <v>2378</v>
       </c>
       <c r="C700" s="15" t="s">
         <v>21</v>
@@ -33541,10 +33541,10 @@
     </row>
     <row r="708" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A708" s="59" t="s">
-        <v>2385</v>
+        <v>2381</v>
       </c>
       <c r="B708" s="14" t="s">
-        <v>2384</v>
+        <v>2380</v>
       </c>
       <c r="C708" s="15" t="s">
         <v>21</v>
@@ -34187,10 +34187,10 @@
     </row>
     <row r="726" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A726" s="59" t="s">
-        <v>2385</v>
+        <v>2381</v>
       </c>
       <c r="B726" s="14" t="s">
-        <v>2384</v>
+        <v>2380</v>
       </c>
       <c r="C726" s="15" t="s">
         <v>21</v>
@@ -34223,10 +34223,10 @@
     </row>
     <row r="727" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A727" s="59" t="s">
-        <v>2383</v>
+        <v>2379</v>
       </c>
       <c r="B727" s="14" t="s">
-        <v>2382</v>
+        <v>2378</v>
       </c>
       <c r="C727" s="15" t="s">
         <v>21</v>
@@ -35414,7 +35414,7 @@
         <v>1245</v>
       </c>
       <c r="B760" s="14" t="s">
-        <v>2386</v>
+        <v>2382</v>
       </c>
       <c r="C760" s="15" t="s">
         <v>21</v>
@@ -37388,7 +37388,7 @@
     <row r="815" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A815" s="13"/>
       <c r="B815" s="14" t="s">
-        <v>2387</v>
+        <v>2383</v>
       </c>
       <c r="C815" s="15" t="s">
         <v>21</v>
@@ -38932,7 +38932,7 @@
     <row r="858" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A858" s="13"/>
       <c r="B858" s="14" t="s">
-        <v>2388</v>
+        <v>2384</v>
       </c>
       <c r="C858" s="15" t="s">
         <v>21</v>
@@ -39398,7 +39398,7 @@
     <row r="871" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A871" s="13"/>
       <c r="B871" s="14" t="s">
-        <v>2394</v>
+        <v>2390</v>
       </c>
       <c r="C871" s="15" t="s">
         <v>21</v>
@@ -41342,7 +41342,7 @@
         <v>2277</v>
       </c>
       <c r="B925" s="14" t="s">
-        <v>2376</v>
+        <v>2372</v>
       </c>
       <c r="C925" s="15" t="s">
         <v>21</v>
@@ -42304,7 +42304,7 @@
     <row r="952" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A952" s="13"/>
       <c r="B952" s="14" t="s">
-        <v>2381</v>
+        <v>2377</v>
       </c>
       <c r="C952" s="15" t="s">
         <v>21</v>
@@ -43274,7 +43274,7 @@
     <row r="979" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A979" s="13"/>
       <c r="B979" s="14" t="s">
-        <v>2389</v>
+        <v>2385</v>
       </c>
       <c r="C979" s="15" t="s">
         <v>21</v>
@@ -45680,7 +45680,7 @@
     <row r="1046" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A1046" s="13"/>
       <c r="B1046" s="14" t="s">
-        <v>2397</v>
+        <v>2393</v>
       </c>
       <c r="C1046" s="15" t="s">
         <v>21</v>
@@ -45714,7 +45714,7 @@
     <row r="1047" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A1047" s="13"/>
       <c r="B1047" s="14" t="s">
-        <v>2398</v>
+        <v>2394</v>
       </c>
       <c r="C1047" s="15" t="s">
         <v>21</v>
@@ -47152,7 +47152,7 @@
     <row r="1087" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A1087" s="13"/>
       <c r="B1087" s="14" t="s">
-        <v>2360</v>
+        <v>2356</v>
       </c>
       <c r="C1087" s="15" t="s">
         <v>21</v>
@@ -47293,10 +47293,10 @@
     </row>
     <row r="1091" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A1091" s="60" t="s">
-        <v>2363</v>
+        <v>2359</v>
       </c>
       <c r="B1091" s="14" t="s">
-        <v>2361</v>
+        <v>2357</v>
       </c>
       <c r="C1091" s="15" t="s">
         <v>21</v>
@@ -47321,7 +47321,7 @@
         <v>1709</v>
       </c>
       <c r="J1091" s="15" t="s">
-        <v>2362</v>
+        <v>2358</v>
       </c>
       <c r="K1091" s="18">
         <v>46117</v>
@@ -50708,10 +50708,10 @@
     </row>
     <row r="1186" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A1186" s="60" t="s">
-        <v>2375</v>
+        <v>2371</v>
       </c>
       <c r="B1186" s="14" t="s">
-        <v>2374</v>
+        <v>2370</v>
       </c>
       <c r="C1186" s="15" t="s">
         <v>21</v>
@@ -54699,7 +54699,7 @@
     <row r="1297" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A1297" s="13"/>
       <c r="B1297" s="14" t="s">
-        <v>2392</v>
+        <v>2388</v>
       </c>
       <c r="C1297" s="15" t="s">
         <v>21</v>
@@ -56245,7 +56245,7 @@
     <row r="1340" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A1340" s="13"/>
       <c r="B1340" s="62" t="s">
-        <v>2390</v>
+        <v>2386</v>
       </c>
       <c r="C1340" s="15" t="s">
         <v>21</v>
@@ -57574,10 +57574,10 @@
     </row>
     <row r="1377" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A1377" s="60" t="s">
-        <v>2367</v>
+        <v>2363</v>
       </c>
       <c r="B1377" s="14" t="s">
-        <v>2365</v>
+        <v>2361</v>
       </c>
       <c r="C1377" s="15" t="s">
         <v>21</v>
@@ -57610,10 +57610,10 @@
     </row>
     <row r="1378" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A1378" s="60" t="s">
-        <v>2368</v>
+        <v>2364</v>
       </c>
       <c r="B1378" s="14" t="s">
-        <v>2366</v>
+        <v>2362</v>
       </c>
       <c r="C1378" s="15" t="s">
         <v>21</v>
@@ -57682,10 +57682,10 @@
     </row>
     <row r="1380" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A1380" s="60" t="s">
-        <v>2370</v>
+        <v>2366</v>
       </c>
       <c r="B1380" s="14" t="s">
-        <v>2369</v>
+        <v>2365</v>
       </c>
       <c r="C1380" s="15" t="s">
         <v>21</v>
@@ -57754,10 +57754,10 @@
     </row>
     <row r="1382" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A1382" s="60" t="s">
-        <v>2372</v>
+        <v>2368</v>
       </c>
       <c r="B1382" s="14" t="s">
-        <v>2371</v>
+        <v>2367</v>
       </c>
       <c r="C1382" s="15" t="s">
         <v>21</v>
@@ -58546,7 +58546,7 @@
     </row>
     <row r="1404" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A1404" s="60" t="s">
-        <v>2373</v>
+        <v>2369</v>
       </c>
       <c r="B1404" s="14" t="s">
         <v>2103</v>
@@ -59087,7 +59087,7 @@
     <row r="1419" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A1419" s="13"/>
       <c r="B1419" s="14" t="s">
-        <v>2391</v>
+        <v>2387</v>
       </c>
       <c r="C1419" s="15" t="s">
         <v>21</v>
@@ -62373,7 +62373,7 @@
         <v>96</v>
       </c>
       <c r="B1511" s="14" t="s">
-        <v>2364</v>
+        <v>2360</v>
       </c>
       <c r="C1511" s="15" t="s">
         <v>21</v>
@@ -64170,10 +64170,10 @@
     </row>
     <row r="1561" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A1561" s="59" t="s">
-        <v>2359</v>
+        <v>2355</v>
       </c>
       <c r="B1561" s="14" t="s">
-        <v>2358</v>
+        <v>2354</v>
       </c>
       <c r="C1561" s="15" t="s">
         <v>21</v>
@@ -65895,7 +65895,7 @@
     <row r="1609" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A1609" s="19"/>
       <c r="B1609" s="20" t="s">
-        <v>2352</v>
+        <v>2395</v>
       </c>
       <c r="C1609" s="21" t="s">
         <v>46</v>
@@ -65914,10 +65914,10 @@
         <v>38</v>
       </c>
       <c r="H1609" s="24" t="s">
+        <v>2352</v>
+      </c>
+      <c r="I1609" s="21" t="s">
         <v>2353</v>
-      </c>
-      <c r="I1609" s="21" t="s">
-        <v>2354</v>
       </c>
       <c r="J1609" s="21">
         <v>6454</v>
@@ -65929,7 +65929,7 @@
     <row r="1610" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A1610" s="19"/>
       <c r="B1610" s="20" t="s">
-        <v>2355</v>
+        <v>2396</v>
       </c>
       <c r="C1610" s="21" t="s">
         <v>46</v>
@@ -65948,10 +65948,10 @@
         <v>38</v>
       </c>
       <c r="H1610" s="24" t="s">
+        <v>2352</v>
+      </c>
+      <c r="I1610" s="21" t="s">
         <v>2353</v>
-      </c>
-      <c r="I1610" s="21" t="s">
-        <v>2354</v>
       </c>
       <c r="J1610" s="21">
         <v>6454</v>
@@ -65963,7 +65963,7 @@
     <row r="1611" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A1611" s="19"/>
       <c r="B1611" s="20" t="s">
-        <v>2356</v>
+        <v>2397</v>
       </c>
       <c r="C1611" s="21" t="s">
         <v>46</v>
@@ -65982,10 +65982,10 @@
         <v>38</v>
       </c>
       <c r="H1611" s="24" t="s">
+        <v>2352</v>
+      </c>
+      <c r="I1611" s="21" t="s">
         <v>2353</v>
-      </c>
-      <c r="I1611" s="21" t="s">
-        <v>2354</v>
       </c>
       <c r="J1611" s="21">
         <v>6454</v>
@@ -65997,7 +65997,7 @@
     <row r="1612" spans="1:11" ht="24.95" customHeight="1" thickTop="1" thickBot="1">
       <c r="A1612" s="19"/>
       <c r="B1612" s="20" t="s">
-        <v>2357</v>
+        <v>2398</v>
       </c>
       <c r="C1612" s="21" t="s">
         <v>46</v>
@@ -66016,10 +66016,10 @@
         <v>38</v>
       </c>
       <c r="H1612" s="24" t="s">
+        <v>2352</v>
+      </c>
+      <c r="I1612" s="21" t="s">
         <v>2353</v>
-      </c>
-      <c r="I1612" s="21" t="s">
-        <v>2354</v>
       </c>
       <c r="J1612" s="21">
         <v>6454</v>

</xml_diff>

<commit_message>
Update all.xlsx with revised transaction data
</commit_message>
<xml_diff>
--- a/data/transactions/all.xlsx
+++ b/data/transactions/all.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24332"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0240706-55E0-443F-BA93-F7241DF4FDDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF2D943C-3A61-4F88-9454-38EF4E332D7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8586" uniqueCount="2399">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8586" uniqueCount="2400">
   <si>
     <t>كود الصنف</t>
   </si>
@@ -7226,6 +7226,9 @@
   </si>
   <si>
     <t>بروفيل باب ثلاجة PVC موديل A144</t>
+  </si>
+  <si>
+    <t>10106023</t>
   </si>
 </sst>
 </file>
@@ -57210,7 +57213,7 @@
     </row>
     <row r="1367" spans="1:11" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1367" s="19" t="s">
-        <v>162</v>
+        <v>2399</v>
       </c>
       <c r="B1367" s="20" t="s">
         <v>2054</v>

</xml_diff>

<commit_message>
Update all.xlsx with new transaction data
</commit_message>
<xml_diff>
--- a/data/transactions/all.xlsx
+++ b/data/transactions/all.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24332"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF2D943C-3A61-4F88-9454-38EF4E332D7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B51B67B4-97C1-4057-910D-73BAFDAEA52D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -50354,7 +50354,7 @@
         <v>1829</v>
       </c>
       <c r="C1176" s="21" t="s">
-        <v>21</v>
+        <v>62</v>
       </c>
       <c r="D1176" s="22">
         <v>1</v>

</xml_diff>

<commit_message>
Update all.xlsx file with additional transaction data revisions
</commit_message>
<xml_diff>
--- a/data/transactions/all.xlsx
+++ b/data/transactions/all.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24332"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DEC0CB7-DC11-43CC-A8E4-5220CA38E0DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F3D222C-AE0A-4659-98F5-8DE72A8D831C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9259" uniqueCount="2581">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9258" uniqueCount="2581">
   <si>
     <t>كود الصنف</t>
   </si>
@@ -7781,7 +7781,7 @@
   <numFmts count="1">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -7852,12 +7852,6 @@
     </font>
     <font>
       <sz val="8"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="18"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -7994,7 +7988,7 @@
     <xf numFmtId="12" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -8012,7 +8006,7 @@
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="13" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="12" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -8024,8 +8018,8 @@
     <xf numFmtId="14" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -8037,11 +8031,11 @@
     <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="2" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="6" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="6" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -8327,7 +8321,7 @@
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.42578125" style="23" customWidth="1"/>
-    <col min="2" max="2" width="52.140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="52.140625" style="34" customWidth="1"/>
     <col min="3" max="3" width="7.85546875" style="1" customWidth="1"/>
     <col min="4" max="4" width="12" style="2" customWidth="1"/>
     <col min="5" max="5" width="15.7109375" style="2" customWidth="1"/>
@@ -66556,7 +66550,7 @@
       <c r="A1621" s="30" t="s">
         <v>2418</v>
       </c>
-      <c r="B1621" s="33" t="s">
+      <c r="B1621" s="8" t="s">
         <v>2419</v>
       </c>
       <c r="C1621" s="7" t="s">
@@ -66589,9 +66583,7 @@
       </c>
     </row>
     <row r="1622" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1622" s="30" t="s">
-        <v>2377</v>
-      </c>
+      <c r="A1622" s="30"/>
       <c r="B1622" s="7" t="s">
         <v>1534</v>
       </c>
@@ -68102,7 +68094,7 @@
         <v>834</v>
       </c>
       <c r="C1664" s="7" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="D1664" s="8">
         <v>2</v>
@@ -69387,11 +69379,10 @@
       </c>
     </row>
     <row r="1700" spans="1:11" ht="22.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B1700" s="20"/>
       <c r="C1700" s="20"/>
       <c r="D1700" s="21"/>
       <c r="E1700" s="21"/>
-      <c r="F1700" s="34">
+      <c r="F1700" s="33">
         <f>SUM(F2:F1699)</f>
         <v>27668891.124196012</v>
       </c>

</xml_diff>

<commit_message>
Update all.xlsx file with the correct supplier names
</commit_message>
<xml_diff>
--- a/data/transactions/all.xlsx
+++ b/data/transactions/all.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24332"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6069646E-B212-4C28-BD86-905E2D0152C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB866F8F-3AC0-47F0-B6CA-86F5AB4C425A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9258" uniqueCount="2581">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9258" uniqueCount="2580">
   <si>
     <t>كود الصنف</t>
   </si>
@@ -7235,9 +7235,6 @@
   </si>
   <si>
     <t>11-2-2026</t>
-  </si>
-  <si>
-    <t>الورشه الفنيه</t>
   </si>
   <si>
     <t>6224</t>
@@ -9200,7 +9197,7 @@
         <v>72</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="C25" s="7" t="s">
         <v>62</v>
@@ -13843,7 +13840,7 @@
         <v>72</v>
       </c>
       <c r="B154" s="7" t="s">
-        <v>2580</v>
+        <v>2579</v>
       </c>
       <c r="C154" s="7" t="s">
         <v>21</v>
@@ -38316,7 +38313,7 @@
         <v>11576</v>
       </c>
       <c r="G834" s="7" t="s">
-        <v>2576</v>
+        <v>2575</v>
       </c>
       <c r="H834" s="10" t="s">
         <v>1391</v>
@@ -42270,7 +42267,7 @@
         <v>7800</v>
       </c>
       <c r="G944" s="7" t="s">
-        <v>2577</v>
+        <v>2576</v>
       </c>
       <c r="H944" s="10">
         <v>46057</v>
@@ -66285,21 +66282,21 @@
         <v>2401</v>
       </c>
       <c r="I1613" s="7" t="s">
+        <v>2397</v>
+      </c>
+      <c r="J1613" s="7" t="s">
         <v>2402</v>
       </c>
-      <c r="J1613" s="7" t="s">
+      <c r="K1613" s="10" t="s">
         <v>2403</v>
-      </c>
-      <c r="K1613" s="10" t="s">
-        <v>2404</v>
       </c>
     </row>
     <row r="1614" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1614" s="30" t="s">
+        <v>2404</v>
+      </c>
+      <c r="B1614" s="7" t="s">
         <v>2405</v>
-      </c>
-      <c r="B1614" s="7" t="s">
-        <v>2406</v>
       </c>
       <c r="C1614" s="7" t="s">
         <v>21</v>
@@ -66321,21 +66318,21 @@
         <v>2401</v>
       </c>
       <c r="I1614" s="7" t="s">
+        <v>2397</v>
+      </c>
+      <c r="J1614" s="7" t="s">
         <v>2402</v>
       </c>
-      <c r="J1614" s="7" t="s">
+      <c r="K1614" s="10" t="s">
         <v>2403</v>
-      </c>
-      <c r="K1614" s="10" t="s">
-        <v>2404</v>
       </c>
     </row>
     <row r="1615" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1615" s="30" t="s">
+        <v>2406</v>
+      </c>
+      <c r="B1615" s="7" t="s">
         <v>2407</v>
-      </c>
-      <c r="B1615" s="7" t="s">
-        <v>2408</v>
       </c>
       <c r="C1615" s="7" t="s">
         <v>21</v>
@@ -66357,13 +66354,13 @@
         <v>2401</v>
       </c>
       <c r="I1615" s="7" t="s">
+        <v>2397</v>
+      </c>
+      <c r="J1615" s="7" t="s">
         <v>2402</v>
       </c>
-      <c r="J1615" s="7" t="s">
+      <c r="K1615" s="10" t="s">
         <v>2403</v>
-      </c>
-      <c r="K1615" s="10" t="s">
-        <v>2404</v>
       </c>
     </row>
     <row r="1616" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -66371,7 +66368,7 @@
         <v>1559</v>
       </c>
       <c r="B1616" s="7" t="s">
-        <v>2409</v>
+        <v>2408</v>
       </c>
       <c r="C1616" s="7" t="s">
         <v>21</v>
@@ -66393,21 +66390,21 @@
         <v>2401</v>
       </c>
       <c r="I1616" s="7" t="s">
+        <v>2397</v>
+      </c>
+      <c r="J1616" s="7" t="s">
         <v>2402</v>
       </c>
-      <c r="J1616" s="7" t="s">
+      <c r="K1616" s="10" t="s">
         <v>2403</v>
-      </c>
-      <c r="K1616" s="10" t="s">
-        <v>2404</v>
       </c>
     </row>
     <row r="1617" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1617" s="30" t="s">
+        <v>2409</v>
+      </c>
+      <c r="B1617" s="7" t="s">
         <v>2410</v>
-      </c>
-      <c r="B1617" s="7" t="s">
-        <v>2411</v>
       </c>
       <c r="C1617" s="7" t="s">
         <v>21</v>
@@ -66429,21 +66426,21 @@
         <v>2401</v>
       </c>
       <c r="I1617" s="7" t="s">
+        <v>2397</v>
+      </c>
+      <c r="J1617" s="7" t="s">
         <v>2402</v>
       </c>
-      <c r="J1617" s="7" t="s">
+      <c r="K1617" s="10" t="s">
         <v>2403</v>
-      </c>
-      <c r="K1617" s="10" t="s">
-        <v>2404</v>
       </c>
     </row>
     <row r="1618" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1618" s="30" t="s">
+        <v>2411</v>
+      </c>
+      <c r="B1618" s="7" t="s">
         <v>2412</v>
-      </c>
-      <c r="B1618" s="7" t="s">
-        <v>2413</v>
       </c>
       <c r="C1618" s="7" t="s">
         <v>21</v>
@@ -66465,21 +66462,21 @@
         <v>2401</v>
       </c>
       <c r="I1618" s="7" t="s">
+        <v>2397</v>
+      </c>
+      <c r="J1618" s="7" t="s">
         <v>2402</v>
       </c>
-      <c r="J1618" s="7" t="s">
+      <c r="K1618" s="10" t="s">
         <v>2403</v>
-      </c>
-      <c r="K1618" s="10" t="s">
-        <v>2404</v>
       </c>
     </row>
     <row r="1619" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1619" s="30" t="s">
+        <v>2413</v>
+      </c>
+      <c r="B1619" s="7" t="s">
         <v>2414</v>
-      </c>
-      <c r="B1619" s="7" t="s">
-        <v>2415</v>
       </c>
       <c r="C1619" s="7" t="s">
         <v>21</v>
@@ -66501,13 +66498,13 @@
         <v>2401</v>
       </c>
       <c r="I1619" s="7" t="s">
+        <v>2397</v>
+      </c>
+      <c r="J1619" s="7" t="s">
         <v>2402</v>
       </c>
-      <c r="J1619" s="7" t="s">
+      <c r="K1619" s="10" t="s">
         <v>2403</v>
-      </c>
-      <c r="K1619" s="10" t="s">
-        <v>2404</v>
       </c>
     </row>
     <row r="1620" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -66515,7 +66512,7 @@
         <v>1549</v>
       </c>
       <c r="B1620" s="7" t="s">
-        <v>2416</v>
+        <v>2415</v>
       </c>
       <c r="C1620" s="7" t="s">
         <v>21</v>
@@ -66537,21 +66534,21 @@
         <v>2401</v>
       </c>
       <c r="I1620" s="7" t="s">
+        <v>2397</v>
+      </c>
+      <c r="J1620" s="7" t="s">
         <v>2402</v>
       </c>
-      <c r="J1620" s="7" t="s">
+      <c r="K1620" s="10" t="s">
         <v>2403</v>
-      </c>
-      <c r="K1620" s="10" t="s">
-        <v>2404</v>
       </c>
     </row>
     <row r="1621" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1621" s="30" t="s">
+        <v>2417</v>
+      </c>
+      <c r="B1621" s="8" t="s">
         <v>2418</v>
-      </c>
-      <c r="B1621" s="8" t="s">
-        <v>2419</v>
       </c>
       <c r="C1621" s="7" t="s">
         <v>21</v>
@@ -66567,16 +66564,16 @@
         <v>4914</v>
       </c>
       <c r="G1621" s="7" t="s">
+        <v>2419</v>
+      </c>
+      <c r="H1621" s="10" t="s">
         <v>2420</v>
       </c>
-      <c r="H1621" s="10" t="s">
+      <c r="I1621" s="7" t="s">
+        <v>2416</v>
+      </c>
+      <c r="J1621" s="7" t="s">
         <v>2421</v>
-      </c>
-      <c r="I1621" s="7" t="s">
-        <v>2417</v>
-      </c>
-      <c r="J1621" s="7" t="s">
-        <v>2422</v>
       </c>
       <c r="K1621" s="10" t="s">
         <v>1153</v>
@@ -66618,7 +66615,7 @@
     </row>
     <row r="1623" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1623" s="30" t="s">
-        <v>2423</v>
+        <v>2422</v>
       </c>
       <c r="B1623" s="7" t="s">
         <v>1535</v>
@@ -66654,10 +66651,10 @@
     </row>
     <row r="1624" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1624" s="30" t="s">
+        <v>2423</v>
+      </c>
+      <c r="B1624" s="7" t="s">
         <v>2424</v>
-      </c>
-      <c r="B1624" s="7" t="s">
-        <v>2425</v>
       </c>
       <c r="C1624" s="7" t="s">
         <v>21</v>
@@ -66673,27 +66670,27 @@
         <v>4030</v>
       </c>
       <c r="G1624" s="7" t="s">
+        <v>2425</v>
+      </c>
+      <c r="H1624" s="10" t="s">
         <v>2426</v>
       </c>
-      <c r="H1624" s="10" t="s">
+      <c r="I1624" s="7" t="s">
         <v>2427</v>
       </c>
-      <c r="I1624" s="7" t="s">
+      <c r="J1624" s="7" t="s">
         <v>2428</v>
       </c>
-      <c r="J1624" s="7" t="s">
+      <c r="K1624" s="10" t="s">
         <v>2429</v>
-      </c>
-      <c r="K1624" s="10" t="s">
-        <v>2430</v>
       </c>
     </row>
     <row r="1625" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1625" s="30" t="s">
+        <v>2430</v>
+      </c>
+      <c r="B1625" s="7" t="s">
         <v>2431</v>
-      </c>
-      <c r="B1625" s="7" t="s">
-        <v>2432</v>
       </c>
       <c r="C1625" s="7" t="s">
         <v>46</v>
@@ -66709,19 +66706,19 @@
         <v>7000</v>
       </c>
       <c r="G1625" s="7" t="s">
+        <v>2425</v>
+      </c>
+      <c r="H1625" s="10" t="s">
         <v>2426</v>
       </c>
-      <c r="H1625" s="10" t="s">
+      <c r="I1625" s="7" t="s">
         <v>2427</v>
       </c>
-      <c r="I1625" s="7" t="s">
+      <c r="J1625" s="7" t="s">
         <v>2428</v>
       </c>
-      <c r="J1625" s="7" t="s">
+      <c r="K1625" s="10" t="s">
         <v>2429</v>
-      </c>
-      <c r="K1625" s="10" t="s">
-        <v>2430</v>
       </c>
     </row>
     <row r="1626" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -66729,7 +66726,7 @@
         <v>609</v>
       </c>
       <c r="B1626" s="7" t="s">
-        <v>2433</v>
+        <v>2432</v>
       </c>
       <c r="C1626" s="7" t="s">
         <v>21</v>
@@ -66745,19 +66742,19 @@
         <v>606315</v>
       </c>
       <c r="G1626" s="7" t="s">
-        <v>2434</v>
+        <v>2433</v>
       </c>
       <c r="H1626" s="10" t="s">
         <v>1783</v>
       </c>
       <c r="I1626" s="7" t="s">
+        <v>2434</v>
+      </c>
+      <c r="J1626" s="7" t="s">
         <v>2435</v>
       </c>
-      <c r="J1626" s="7" t="s">
+      <c r="K1626" s="10" t="s">
         <v>2436</v>
-      </c>
-      <c r="K1626" s="10" t="s">
-        <v>2437</v>
       </c>
     </row>
     <row r="1627" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -66765,7 +66762,7 @@
         <v>1737</v>
       </c>
       <c r="B1627" s="7" t="s">
-        <v>2438</v>
+        <v>2437</v>
       </c>
       <c r="C1627" s="7" t="s">
         <v>21</v>
@@ -66781,19 +66778,19 @@
         <v>227368.08</v>
       </c>
       <c r="G1627" s="7" t="s">
-        <v>2434</v>
+        <v>2433</v>
       </c>
       <c r="H1627" s="10" t="s">
         <v>1783</v>
       </c>
       <c r="I1627" s="7" t="s">
+        <v>2434</v>
+      </c>
+      <c r="J1627" s="7" t="s">
         <v>2435</v>
       </c>
-      <c r="J1627" s="7" t="s">
+      <c r="K1627" s="10" t="s">
         <v>2436</v>
-      </c>
-      <c r="K1627" s="10" t="s">
-        <v>2437</v>
       </c>
     </row>
     <row r="1628" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -66801,7 +66798,7 @@
         <v>577</v>
       </c>
       <c r="B1628" s="7" t="s">
-        <v>2439</v>
+        <v>2438</v>
       </c>
       <c r="C1628" s="7" t="s">
         <v>21</v>
@@ -66817,27 +66814,27 @@
         <v>137369.81</v>
       </c>
       <c r="G1628" s="7" t="s">
-        <v>2434</v>
+        <v>2433</v>
       </c>
       <c r="H1628" s="10" t="s">
         <v>1783</v>
       </c>
       <c r="I1628" s="7" t="s">
+        <v>2434</v>
+      </c>
+      <c r="J1628" s="7" t="s">
         <v>2435</v>
       </c>
-      <c r="J1628" s="7" t="s">
+      <c r="K1628" s="10" t="s">
         <v>2436</v>
-      </c>
-      <c r="K1628" s="10" t="s">
-        <v>2437</v>
       </c>
     </row>
     <row r="1629" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1629" s="30" t="s">
+        <v>2439</v>
+      </c>
+      <c r="B1629" s="7" t="s">
         <v>2440</v>
-      </c>
-      <c r="B1629" s="7" t="s">
-        <v>2441</v>
       </c>
       <c r="C1629" s="7" t="s">
         <v>21</v>
@@ -66853,7 +66850,7 @@
         <v>3750</v>
       </c>
       <c r="G1629" s="7" t="s">
-        <v>2442</v>
+        <v>2441</v>
       </c>
       <c r="H1629" s="10" t="s">
         <v>1789</v>
@@ -66862,7 +66859,7 @@
         <v>534</v>
       </c>
       <c r="J1629" s="7" t="s">
-        <v>2443</v>
+        <v>2442</v>
       </c>
       <c r="K1629" s="10" t="s">
         <v>1793</v>
@@ -66870,10 +66867,10 @@
     </row>
     <row r="1630" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1630" s="30" t="s">
+        <v>2443</v>
+      </c>
+      <c r="B1630" s="7" t="s">
         <v>2444</v>
-      </c>
-      <c r="B1630" s="7" t="s">
-        <v>2445</v>
       </c>
       <c r="C1630" s="7" t="s">
         <v>21</v>
@@ -66889,7 +66886,7 @@
         <v>18750</v>
       </c>
       <c r="G1630" s="7" t="s">
-        <v>2442</v>
+        <v>2441</v>
       </c>
       <c r="H1630" s="10" t="s">
         <v>1789</v>
@@ -66898,7 +66895,7 @@
         <v>534</v>
       </c>
       <c r="J1630" s="7" t="s">
-        <v>2443</v>
+        <v>2442</v>
       </c>
       <c r="K1630" s="10" t="s">
         <v>1793</v>
@@ -66925,7 +66922,7 @@
         <v>18750</v>
       </c>
       <c r="G1631" s="7" t="s">
-        <v>2442</v>
+        <v>2441</v>
       </c>
       <c r="H1631" s="10" t="s">
         <v>1789</v>
@@ -66934,7 +66931,7 @@
         <v>534</v>
       </c>
       <c r="J1631" s="7" t="s">
-        <v>2443</v>
+        <v>2442</v>
       </c>
       <c r="K1631" s="10" t="s">
         <v>1793</v>
@@ -66942,10 +66939,10 @@
     </row>
     <row r="1632" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1632" s="30" t="s">
+        <v>2445</v>
+      </c>
+      <c r="B1632" s="7" t="s">
         <v>2446</v>
-      </c>
-      <c r="B1632" s="7" t="s">
-        <v>2447</v>
       </c>
       <c r="C1632" s="7" t="s">
         <v>21</v>
@@ -66961,7 +66958,7 @@
         <v>300</v>
       </c>
       <c r="G1632" s="7" t="s">
-        <v>2442</v>
+        <v>2441</v>
       </c>
       <c r="H1632" s="10" t="s">
         <v>1789</v>
@@ -66970,7 +66967,7 @@
         <v>534</v>
       </c>
       <c r="J1632" s="7" t="s">
-        <v>2443</v>
+        <v>2442</v>
       </c>
       <c r="K1632" s="10" t="s">
         <v>1793</v>
@@ -66978,10 +66975,10 @@
     </row>
     <row r="1633" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1633" s="30" t="s">
+        <v>2447</v>
+      </c>
+      <c r="B1633" s="7" t="s">
         <v>2448</v>
-      </c>
-      <c r="B1633" s="7" t="s">
-        <v>2449</v>
       </c>
       <c r="C1633" s="7" t="s">
         <v>21</v>
@@ -66997,7 +66994,7 @@
         <v>200</v>
       </c>
       <c r="G1633" s="7" t="s">
-        <v>2442</v>
+        <v>2441</v>
       </c>
       <c r="H1633" s="10" t="s">
         <v>1789</v>
@@ -67006,7 +67003,7 @@
         <v>534</v>
       </c>
       <c r="J1633" s="7" t="s">
-        <v>2443</v>
+        <v>2442</v>
       </c>
       <c r="K1633" s="10" t="s">
         <v>1793</v>
@@ -67014,10 +67011,10 @@
     </row>
     <row r="1634" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1634" s="30" t="s">
+        <v>2449</v>
+      </c>
+      <c r="B1634" s="7" t="s">
         <v>2450</v>
-      </c>
-      <c r="B1634" s="7" t="s">
-        <v>2451</v>
       </c>
       <c r="C1634" s="7" t="s">
         <v>21</v>
@@ -67033,7 +67030,7 @@
         <v>3375</v>
       </c>
       <c r="G1634" s="7" t="s">
-        <v>2442</v>
+        <v>2441</v>
       </c>
       <c r="H1634" s="10" t="s">
         <v>1789</v>
@@ -67042,7 +67039,7 @@
         <v>534</v>
       </c>
       <c r="J1634" s="7" t="s">
-        <v>2443</v>
+        <v>2442</v>
       </c>
       <c r="K1634" s="10" t="s">
         <v>1793</v>
@@ -67053,7 +67050,7 @@
         <v>537</v>
       </c>
       <c r="B1635" s="7" t="s">
-        <v>2452</v>
+        <v>2451</v>
       </c>
       <c r="C1635" s="7" t="s">
         <v>21</v>
@@ -67069,7 +67066,7 @@
         <v>750</v>
       </c>
       <c r="G1635" s="7" t="s">
-        <v>2442</v>
+        <v>2441</v>
       </c>
       <c r="H1635" s="10" t="s">
         <v>1789</v>
@@ -67078,7 +67075,7 @@
         <v>534</v>
       </c>
       <c r="J1635" s="7" t="s">
-        <v>2443</v>
+        <v>2442</v>
       </c>
       <c r="K1635" s="10" t="s">
         <v>1793</v>
@@ -67086,10 +67083,10 @@
     </row>
     <row r="1636" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1636" s="30" t="s">
+        <v>2452</v>
+      </c>
+      <c r="B1636" s="7" t="s">
         <v>2453</v>
-      </c>
-      <c r="B1636" s="7" t="s">
-        <v>2454</v>
       </c>
       <c r="C1636" s="7" t="s">
         <v>21</v>
@@ -67105,7 +67102,7 @@
         <v>1500</v>
       </c>
       <c r="G1636" s="7" t="s">
-        <v>2442</v>
+        <v>2441</v>
       </c>
       <c r="H1636" s="10" t="s">
         <v>1789</v>
@@ -67114,7 +67111,7 @@
         <v>534</v>
       </c>
       <c r="J1636" s="7" t="s">
-        <v>2443</v>
+        <v>2442</v>
       </c>
       <c r="K1636" s="10" t="s">
         <v>1793</v>
@@ -67122,10 +67119,10 @@
     </row>
     <row r="1637" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1637" s="30" t="s">
+        <v>2454</v>
+      </c>
+      <c r="B1637" s="7" t="s">
         <v>2455</v>
-      </c>
-      <c r="B1637" s="7" t="s">
-        <v>2456</v>
       </c>
       <c r="C1637" s="7" t="s">
         <v>21</v>
@@ -67141,7 +67138,7 @@
         <v>4800</v>
       </c>
       <c r="G1637" s="7" t="s">
-        <v>2442</v>
+        <v>2441</v>
       </c>
       <c r="H1637" s="10" t="s">
         <v>1789</v>
@@ -67150,7 +67147,7 @@
         <v>534</v>
       </c>
       <c r="J1637" s="7" t="s">
-        <v>2443</v>
+        <v>2442</v>
       </c>
       <c r="K1637" s="10" t="s">
         <v>1793</v>
@@ -67177,7 +67174,7 @@
         <v>1250</v>
       </c>
       <c r="G1638" s="7" t="s">
-        <v>2442</v>
+        <v>2441</v>
       </c>
       <c r="H1638" s="10" t="s">
         <v>1789</v>
@@ -67186,7 +67183,7 @@
         <v>534</v>
       </c>
       <c r="J1638" s="7" t="s">
-        <v>2443</v>
+        <v>2442</v>
       </c>
       <c r="K1638" s="10" t="s">
         <v>1793</v>
@@ -67197,7 +67194,7 @@
         <v>847</v>
       </c>
       <c r="B1639" s="7" t="s">
-        <v>2457</v>
+        <v>2456</v>
       </c>
       <c r="C1639" s="7" t="s">
         <v>21</v>
@@ -67213,7 +67210,7 @@
         <v>5625</v>
       </c>
       <c r="G1639" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1639" s="10" t="s">
         <v>1789</v>
@@ -67222,7 +67219,7 @@
         <v>534</v>
       </c>
       <c r="J1639" s="7" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
       <c r="K1639" s="10" t="s">
         <v>1793</v>
@@ -67230,10 +67227,10 @@
     </row>
     <row r="1640" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1640" s="30" t="s">
+        <v>2459</v>
+      </c>
+      <c r="B1640" s="7" t="s">
         <v>2460</v>
-      </c>
-      <c r="B1640" s="7" t="s">
-        <v>2461</v>
       </c>
       <c r="C1640" s="7" t="s">
         <v>46</v>
@@ -67249,7 +67246,7 @@
         <v>2250</v>
       </c>
       <c r="G1640" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1640" s="10" t="s">
         <v>1789</v>
@@ -67258,7 +67255,7 @@
         <v>534</v>
       </c>
       <c r="J1640" s="7" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
       <c r="K1640" s="10" t="s">
         <v>1793</v>
@@ -67266,10 +67263,10 @@
     </row>
     <row r="1641" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1641" s="30" t="s">
+        <v>2461</v>
+      </c>
+      <c r="B1641" s="7" t="s">
         <v>2462</v>
-      </c>
-      <c r="B1641" s="7" t="s">
-        <v>2463</v>
       </c>
       <c r="C1641" s="7" t="s">
         <v>21</v>
@@ -67285,7 +67282,7 @@
         <v>2250</v>
       </c>
       <c r="G1641" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1641" s="10" t="s">
         <v>1789</v>
@@ -67294,7 +67291,7 @@
         <v>534</v>
       </c>
       <c r="J1641" s="7" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
       <c r="K1641" s="10" t="s">
         <v>1793</v>
@@ -67302,10 +67299,10 @@
     </row>
     <row r="1642" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1642" s="30" t="s">
+        <v>2463</v>
+      </c>
+      <c r="B1642" s="7" t="s">
         <v>2464</v>
-      </c>
-      <c r="B1642" s="7" t="s">
-        <v>2465</v>
       </c>
       <c r="C1642" s="7" t="s">
         <v>21</v>
@@ -67321,7 +67318,7 @@
         <v>575</v>
       </c>
       <c r="G1642" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1642" s="10" t="s">
         <v>1789</v>
@@ -67330,7 +67327,7 @@
         <v>534</v>
       </c>
       <c r="J1642" s="7" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
       <c r="K1642" s="10" t="s">
         <v>1793</v>
@@ -67338,7 +67335,7 @@
     </row>
     <row r="1643" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1643" s="30" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
       <c r="B1643" s="7" t="s">
         <v>2065</v>
@@ -67357,7 +67354,7 @@
         <v>500</v>
       </c>
       <c r="G1643" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1643" s="10" t="s">
         <v>1789</v>
@@ -67366,7 +67363,7 @@
         <v>534</v>
       </c>
       <c r="J1643" s="7" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
       <c r="K1643" s="10" t="s">
         <v>1793</v>
@@ -67374,10 +67371,10 @@
     </row>
     <row r="1644" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1644" s="30" t="s">
+        <v>2452</v>
+      </c>
+      <c r="B1644" s="7" t="s">
         <v>2453</v>
-      </c>
-      <c r="B1644" s="7" t="s">
-        <v>2454</v>
       </c>
       <c r="C1644" s="7" t="s">
         <v>21</v>
@@ -67393,7 +67390,7 @@
         <v>90</v>
       </c>
       <c r="G1644" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1644" s="10" t="s">
         <v>1789</v>
@@ -67402,7 +67399,7 @@
         <v>534</v>
       </c>
       <c r="J1644" s="7" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
       <c r="K1644" s="10" t="s">
         <v>1793</v>
@@ -67410,10 +67407,10 @@
     </row>
     <row r="1645" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1645" s="30" t="s">
+        <v>2466</v>
+      </c>
+      <c r="B1645" s="7" t="s">
         <v>2467</v>
-      </c>
-      <c r="B1645" s="7" t="s">
-        <v>2468</v>
       </c>
       <c r="C1645" s="7" t="s">
         <v>21</v>
@@ -67429,7 +67426,7 @@
         <v>675</v>
       </c>
       <c r="G1645" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1645" s="10" t="s">
         <v>1789</v>
@@ -67438,7 +67435,7 @@
         <v>534</v>
       </c>
       <c r="J1645" s="7" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
       <c r="K1645" s="10" t="s">
         <v>1793</v>
@@ -67446,10 +67443,10 @@
     </row>
     <row r="1646" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1646" s="30" t="s">
+        <v>2468</v>
+      </c>
+      <c r="B1646" s="7" t="s">
         <v>2469</v>
-      </c>
-      <c r="B1646" s="7" t="s">
-        <v>2470</v>
       </c>
       <c r="C1646" s="7" t="s">
         <v>21</v>
@@ -67465,7 +67462,7 @@
         <v>11000</v>
       </c>
       <c r="G1646" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1646" s="10" t="s">
         <v>1789</v>
@@ -67474,7 +67471,7 @@
         <v>534</v>
       </c>
       <c r="J1646" s="7" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
       <c r="K1646" s="10" t="s">
         <v>1793</v>
@@ -67485,7 +67482,7 @@
         <v>535</v>
       </c>
       <c r="B1647" s="7" t="s">
-        <v>2471</v>
+        <v>2470</v>
       </c>
       <c r="C1647" s="7" t="s">
         <v>21</v>
@@ -67501,7 +67498,7 @@
         <v>300</v>
       </c>
       <c r="G1647" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1647" s="10" t="s">
         <v>1789</v>
@@ -67510,7 +67507,7 @@
         <v>534</v>
       </c>
       <c r="J1647" s="7" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
       <c r="K1647" s="10" t="s">
         <v>1793</v>
@@ -67518,10 +67515,10 @@
     </row>
     <row r="1648" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1648" s="30" t="s">
+        <v>2471</v>
+      </c>
+      <c r="B1648" s="7" t="s">
         <v>2472</v>
-      </c>
-      <c r="B1648" s="7" t="s">
-        <v>2473</v>
       </c>
       <c r="C1648" s="7" t="s">
         <v>21</v>
@@ -67537,7 +67534,7 @@
         <v>300</v>
       </c>
       <c r="G1648" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1648" s="10" t="s">
         <v>1789</v>
@@ -67546,7 +67543,7 @@
         <v>534</v>
       </c>
       <c r="J1648" s="7" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
       <c r="K1648" s="10" t="s">
         <v>1793</v>
@@ -67554,10 +67551,10 @@
     </row>
     <row r="1649" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1649" s="30" t="s">
+        <v>2473</v>
+      </c>
+      <c r="B1649" s="7" t="s">
         <v>2474</v>
-      </c>
-      <c r="B1649" s="7" t="s">
-        <v>2475</v>
       </c>
       <c r="C1649" s="7" t="s">
         <v>21</v>
@@ -67573,7 +67570,7 @@
         <v>150</v>
       </c>
       <c r="G1649" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1649" s="10" t="s">
         <v>1789</v>
@@ -67582,7 +67579,7 @@
         <v>534</v>
       </c>
       <c r="J1649" s="7" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
       <c r="K1649" s="10" t="s">
         <v>1793</v>
@@ -67590,10 +67587,10 @@
     </row>
     <row r="1650" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1650" s="30" t="s">
+        <v>2475</v>
+      </c>
+      <c r="B1650" s="7" t="s">
         <v>2476</v>
-      </c>
-      <c r="B1650" s="7" t="s">
-        <v>2477</v>
       </c>
       <c r="C1650" s="7" t="s">
         <v>21</v>
@@ -67609,7 +67606,7 @@
         <v>275</v>
       </c>
       <c r="G1650" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1650" s="10" t="s">
         <v>1789</v>
@@ -67618,7 +67615,7 @@
         <v>534</v>
       </c>
       <c r="J1650" s="7" t="s">
-        <v>2478</v>
+        <v>2477</v>
       </c>
       <c r="K1650" s="10" t="s">
         <v>1793</v>
@@ -67626,10 +67623,10 @@
     </row>
     <row r="1651" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1651" s="30" t="s">
+        <v>2478</v>
+      </c>
+      <c r="B1651" s="7" t="s">
         <v>2479</v>
-      </c>
-      <c r="B1651" s="7" t="s">
-        <v>2480</v>
       </c>
       <c r="C1651" s="7" t="s">
         <v>21</v>
@@ -67645,7 +67642,7 @@
         <v>3000</v>
       </c>
       <c r="G1651" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1651" s="10" t="s">
         <v>1789</v>
@@ -67654,7 +67651,7 @@
         <v>534</v>
       </c>
       <c r="J1651" s="7" t="s">
-        <v>2478</v>
+        <v>2477</v>
       </c>
       <c r="K1651" s="10" t="s">
         <v>1793</v>
@@ -67662,10 +67659,10 @@
     </row>
     <row r="1652" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1652" s="30" t="s">
-        <v>2578</v>
+        <v>2577</v>
       </c>
       <c r="B1652" s="7" t="s">
-        <v>2482</v>
+        <v>2481</v>
       </c>
       <c r="C1652" s="7" t="s">
         <v>21</v>
@@ -67681,7 +67678,7 @@
         <v>1500</v>
       </c>
       <c r="G1652" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1652" s="10" t="s">
         <v>1789</v>
@@ -67690,7 +67687,7 @@
         <v>534</v>
       </c>
       <c r="J1652" s="7" t="s">
-        <v>2478</v>
+        <v>2477</v>
       </c>
       <c r="K1652" s="10" t="s">
         <v>1793</v>
@@ -67698,10 +67695,10 @@
     </row>
     <row r="1653" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1653" s="30" t="s">
+        <v>2482</v>
+      </c>
+      <c r="B1653" s="7" t="s">
         <v>2483</v>
-      </c>
-      <c r="B1653" s="7" t="s">
-        <v>2484</v>
       </c>
       <c r="C1653" s="7" t="s">
         <v>21</v>
@@ -67717,7 +67714,7 @@
         <v>100</v>
       </c>
       <c r="G1653" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1653" s="10" t="s">
         <v>1789</v>
@@ -67726,7 +67723,7 @@
         <v>534</v>
       </c>
       <c r="J1653" s="7" t="s">
-        <v>2478</v>
+        <v>2477</v>
       </c>
       <c r="K1653" s="10" t="s">
         <v>1793</v>
@@ -67734,10 +67731,10 @@
     </row>
     <row r="1654" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1654" s="30" t="s">
+        <v>2484</v>
+      </c>
+      <c r="B1654" s="7" t="s">
         <v>2485</v>
-      </c>
-      <c r="B1654" s="7" t="s">
-        <v>2486</v>
       </c>
       <c r="C1654" s="7" t="s">
         <v>21</v>
@@ -67753,7 +67750,7 @@
         <v>75</v>
       </c>
       <c r="G1654" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1654" s="10" t="s">
         <v>1789</v>
@@ -67762,7 +67759,7 @@
         <v>534</v>
       </c>
       <c r="J1654" s="7" t="s">
-        <v>2478</v>
+        <v>2477</v>
       </c>
       <c r="K1654" s="10" t="s">
         <v>1793</v>
@@ -67770,10 +67767,10 @@
     </row>
     <row r="1655" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1655" s="30" t="s">
+        <v>2486</v>
+      </c>
+      <c r="B1655" s="7" t="s">
         <v>2487</v>
-      </c>
-      <c r="B1655" s="7" t="s">
-        <v>2488</v>
       </c>
       <c r="C1655" s="7" t="s">
         <v>21</v>
@@ -67789,7 +67786,7 @@
         <v>925</v>
       </c>
       <c r="G1655" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1655" s="10" t="s">
         <v>1789</v>
@@ -67798,7 +67795,7 @@
         <v>534</v>
       </c>
       <c r="J1655" s="7" t="s">
-        <v>2478</v>
+        <v>2477</v>
       </c>
       <c r="K1655" s="10" t="s">
         <v>1793</v>
@@ -67806,10 +67803,10 @@
     </row>
     <row r="1656" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1656" s="30" t="s">
+        <v>2488</v>
+      </c>
+      <c r="B1656" s="7" t="s">
         <v>2489</v>
-      </c>
-      <c r="B1656" s="7" t="s">
-        <v>2490</v>
       </c>
       <c r="C1656" s="7" t="s">
         <v>21</v>
@@ -67825,7 +67822,7 @@
         <v>17250</v>
       </c>
       <c r="G1656" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1656" s="10" t="s">
         <v>1789</v>
@@ -67834,7 +67831,7 @@
         <v>534</v>
       </c>
       <c r="J1656" s="7" t="s">
-        <v>2478</v>
+        <v>2477</v>
       </c>
       <c r="K1656" s="10" t="s">
         <v>1793</v>
@@ -67842,10 +67839,10 @@
     </row>
     <row r="1657" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1657" s="30" t="s">
+        <v>2490</v>
+      </c>
+      <c r="B1657" s="7" t="s">
         <v>2491</v>
-      </c>
-      <c r="B1657" s="7" t="s">
-        <v>2492</v>
       </c>
       <c r="C1657" s="7" t="s">
         <v>21</v>
@@ -67861,7 +67858,7 @@
         <v>2250</v>
       </c>
       <c r="G1657" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1657" s="10" t="s">
         <v>1789</v>
@@ -67870,7 +67867,7 @@
         <v>534</v>
       </c>
       <c r="J1657" s="7" t="s">
-        <v>2478</v>
+        <v>2477</v>
       </c>
       <c r="K1657" s="10" t="s">
         <v>1793</v>
@@ -67881,7 +67878,7 @@
         <v>841</v>
       </c>
       <c r="B1658" s="7" t="s">
-        <v>2493</v>
+        <v>2492</v>
       </c>
       <c r="C1658" s="7" t="s">
         <v>21</v>
@@ -67897,7 +67894,7 @@
         <v>70</v>
       </c>
       <c r="G1658" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1658" s="10" t="s">
         <v>1789</v>
@@ -67906,7 +67903,7 @@
         <v>534</v>
       </c>
       <c r="J1658" s="7" t="s">
-        <v>2478</v>
+        <v>2477</v>
       </c>
       <c r="K1658" s="10" t="s">
         <v>1793</v>
@@ -67917,7 +67914,7 @@
         <v>2067</v>
       </c>
       <c r="B1659" s="7" t="s">
-        <v>2494</v>
+        <v>2493</v>
       </c>
       <c r="C1659" s="7" t="s">
         <v>21</v>
@@ -67933,7 +67930,7 @@
         <v>1225</v>
       </c>
       <c r="G1659" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1659" s="10" t="s">
         <v>1789</v>
@@ -67942,7 +67939,7 @@
         <v>534</v>
       </c>
       <c r="J1659" s="7" t="s">
-        <v>2478</v>
+        <v>2477</v>
       </c>
       <c r="K1659" s="10" t="s">
         <v>1793</v>
@@ -67950,10 +67947,10 @@
     </row>
     <row r="1660" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1660" s="30" t="s">
-        <v>2579</v>
+        <v>2578</v>
       </c>
       <c r="B1660" s="7" t="s">
-        <v>2496</v>
+        <v>2495</v>
       </c>
       <c r="C1660" s="7" t="s">
         <v>21</v>
@@ -67969,7 +67966,7 @@
         <v>1750</v>
       </c>
       <c r="G1660" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1660" s="10" t="s">
         <v>1789</v>
@@ -67978,7 +67975,7 @@
         <v>534</v>
       </c>
       <c r="J1660" s="7" t="s">
-        <v>2478</v>
+        <v>2477</v>
       </c>
       <c r="K1660" s="10" t="s">
         <v>1793</v>
@@ -67987,7 +67984,7 @@
     <row r="1661" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1661" s="6"/>
       <c r="B1661" s="7" t="s">
-        <v>2497</v>
+        <v>2496</v>
       </c>
       <c r="C1661" s="7" t="s">
         <v>21</v>
@@ -68003,7 +68000,7 @@
         <v>1540</v>
       </c>
       <c r="G1661" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1661" s="10" t="s">
         <v>1789</v>
@@ -68012,7 +68009,7 @@
         <v>534</v>
       </c>
       <c r="J1661" s="7" t="s">
-        <v>2498</v>
+        <v>2497</v>
       </c>
       <c r="K1661" s="10" t="s">
         <v>1793</v>
@@ -68021,7 +68018,7 @@
     <row r="1662" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1662" s="6"/>
       <c r="B1662" s="7" t="s">
-        <v>2499</v>
+        <v>2498</v>
       </c>
       <c r="C1662" s="7" t="s">
         <v>21</v>
@@ -68037,7 +68034,7 @@
         <v>6125</v>
       </c>
       <c r="G1662" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1662" s="10" t="s">
         <v>1789</v>
@@ -68046,7 +68043,7 @@
         <v>534</v>
       </c>
       <c r="J1662" s="7" t="s">
-        <v>2498</v>
+        <v>2497</v>
       </c>
       <c r="K1662" s="10" t="s">
         <v>1793</v>
@@ -68055,7 +68052,7 @@
     <row r="1663" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1663" s="6"/>
       <c r="B1663" s="7" t="s">
-        <v>2500</v>
+        <v>2499</v>
       </c>
       <c r="C1663" s="7" t="s">
         <v>21</v>
@@ -68071,7 +68068,7 @@
         <v>570</v>
       </c>
       <c r="G1663" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1663" s="10" t="s">
         <v>1789</v>
@@ -68080,7 +68077,7 @@
         <v>534</v>
       </c>
       <c r="J1663" s="7" t="s">
-        <v>2498</v>
+        <v>2497</v>
       </c>
       <c r="K1663" s="10" t="s">
         <v>1793</v>
@@ -68107,7 +68104,7 @@
         <v>250</v>
       </c>
       <c r="G1664" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1664" s="10" t="s">
         <v>1789</v>
@@ -68116,7 +68113,7 @@
         <v>534</v>
       </c>
       <c r="J1664" s="7" t="s">
-        <v>2498</v>
+        <v>2497</v>
       </c>
       <c r="K1664" s="10" t="s">
         <v>1793</v>
@@ -68124,10 +68121,10 @@
     </row>
     <row r="1665" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1665" s="30" t="s">
-        <v>2481</v>
+        <v>2480</v>
       </c>
       <c r="B1665" s="7" t="s">
-        <v>2501</v>
+        <v>2500</v>
       </c>
       <c r="C1665" s="7" t="s">
         <v>713</v>
@@ -68143,7 +68140,7 @@
         <v>5800</v>
       </c>
       <c r="G1665" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1665" s="10" t="s">
         <v>1789</v>
@@ -68152,7 +68149,7 @@
         <v>534</v>
       </c>
       <c r="J1665" s="7" t="s">
-        <v>2498</v>
+        <v>2497</v>
       </c>
       <c r="K1665" s="10" t="s">
         <v>1793</v>
@@ -68160,10 +68157,10 @@
     </row>
     <row r="1666" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1666" s="30" t="s">
-        <v>2495</v>
+        <v>2494</v>
       </c>
       <c r="B1666" s="7" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
       <c r="C1666" s="7" t="s">
         <v>21</v>
@@ -68179,7 +68176,7 @@
         <v>150</v>
       </c>
       <c r="G1666" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1666" s="10" t="s">
         <v>1789</v>
@@ -68188,7 +68185,7 @@
         <v>534</v>
       </c>
       <c r="J1666" s="7" t="s">
-        <v>2498</v>
+        <v>2497</v>
       </c>
       <c r="K1666" s="10" t="s">
         <v>1793</v>
@@ -68196,7 +68193,7 @@
     </row>
     <row r="1667" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1667" s="30" t="s">
-        <v>2503</v>
+        <v>2502</v>
       </c>
       <c r="B1667" s="7" t="s">
         <v>840</v>
@@ -68215,7 +68212,7 @@
         <v>1140</v>
       </c>
       <c r="G1667" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1667" s="10" t="s">
         <v>1789</v>
@@ -68224,7 +68221,7 @@
         <v>534</v>
       </c>
       <c r="J1667" s="7" t="s">
-        <v>2498</v>
+        <v>2497</v>
       </c>
       <c r="K1667" s="10" t="s">
         <v>1793</v>
@@ -68232,10 +68229,10 @@
     </row>
     <row r="1668" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1668" s="30" t="s">
+        <v>2503</v>
+      </c>
+      <c r="B1668" s="7" t="s">
         <v>2504</v>
-      </c>
-      <c r="B1668" s="7" t="s">
-        <v>2505</v>
       </c>
       <c r="C1668" s="7" t="s">
         <v>21</v>
@@ -68251,7 +68248,7 @@
         <v>660</v>
       </c>
       <c r="G1668" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1668" s="10" t="s">
         <v>1789</v>
@@ -68260,7 +68257,7 @@
         <v>534</v>
       </c>
       <c r="J1668" s="7" t="s">
-        <v>2498</v>
+        <v>2497</v>
       </c>
       <c r="K1668" s="10" t="s">
         <v>1793</v>
@@ -68268,7 +68265,7 @@
     </row>
     <row r="1669" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1669" s="30" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="B1669" s="7" t="s">
         <v>2083</v>
@@ -68287,7 +68284,7 @@
         <v>768</v>
       </c>
       <c r="G1669" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1669" s="10" t="s">
         <v>1789</v>
@@ -68296,7 +68293,7 @@
         <v>534</v>
       </c>
       <c r="J1669" s="7" t="s">
-        <v>2498</v>
+        <v>2497</v>
       </c>
       <c r="K1669" s="10" t="s">
         <v>1793</v>
@@ -68304,10 +68301,10 @@
     </row>
     <row r="1670" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1670" s="30" t="s">
+        <v>2506</v>
+      </c>
+      <c r="B1670" s="7" t="s">
         <v>2507</v>
-      </c>
-      <c r="B1670" s="7" t="s">
-        <v>2508</v>
       </c>
       <c r="C1670" s="7" t="s">
         <v>21</v>
@@ -68323,7 +68320,7 @@
         <v>330</v>
       </c>
       <c r="G1670" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1670" s="10" t="s">
         <v>1789</v>
@@ -68332,7 +68329,7 @@
         <v>534</v>
       </c>
       <c r="J1670" s="7" t="s">
-        <v>2498</v>
+        <v>2497</v>
       </c>
       <c r="K1670" s="10" t="s">
         <v>1793</v>
@@ -68340,10 +68337,10 @@
     </row>
     <row r="1671" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1671" s="30" t="s">
+        <v>2508</v>
+      </c>
+      <c r="B1671" s="7" t="s">
         <v>2509</v>
-      </c>
-      <c r="B1671" s="7" t="s">
-        <v>2510</v>
       </c>
       <c r="C1671" s="7" t="s">
         <v>21</v>
@@ -68359,7 +68356,7 @@
         <v>1500</v>
       </c>
       <c r="G1671" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1671" s="10" t="s">
         <v>1789</v>
@@ -68368,7 +68365,7 @@
         <v>534</v>
       </c>
       <c r="J1671" s="7" t="s">
-        <v>2498</v>
+        <v>2497</v>
       </c>
       <c r="K1671" s="10" t="s">
         <v>1793</v>
@@ -68376,10 +68373,10 @@
     </row>
     <row r="1672" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1672" s="30" t="s">
+        <v>2510</v>
+      </c>
+      <c r="B1672" s="7" t="s">
         <v>2511</v>
-      </c>
-      <c r="B1672" s="7" t="s">
-        <v>2512</v>
       </c>
       <c r="C1672" s="7" t="s">
         <v>21</v>
@@ -68395,7 +68392,7 @@
         <v>1200</v>
       </c>
       <c r="G1672" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1672" s="10" t="s">
         <v>1789</v>
@@ -68404,7 +68401,7 @@
         <v>534</v>
       </c>
       <c r="J1672" s="7" t="s">
-        <v>2513</v>
+        <v>2512</v>
       </c>
       <c r="K1672" s="10" t="s">
         <v>1793</v>
@@ -68412,10 +68409,10 @@
     </row>
     <row r="1673" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1673" s="30" t="s">
+        <v>2513</v>
+      </c>
+      <c r="B1673" s="7" t="s">
         <v>2514</v>
-      </c>
-      <c r="B1673" s="7" t="s">
-        <v>2515</v>
       </c>
       <c r="C1673" s="7" t="s">
         <v>21</v>
@@ -68431,7 +68428,7 @@
         <v>500</v>
       </c>
       <c r="G1673" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1673" s="10" t="s">
         <v>1789</v>
@@ -68440,7 +68437,7 @@
         <v>534</v>
       </c>
       <c r="J1673" s="7" t="s">
-        <v>2513</v>
+        <v>2512</v>
       </c>
       <c r="K1673" s="10" t="s">
         <v>1793</v>
@@ -68448,10 +68445,10 @@
     </row>
     <row r="1674" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1674" s="30" t="s">
+        <v>2515</v>
+      </c>
+      <c r="B1674" s="7" t="s">
         <v>2516</v>
-      </c>
-      <c r="B1674" s="7" t="s">
-        <v>2517</v>
       </c>
       <c r="C1674" s="7" t="s">
         <v>21</v>
@@ -68467,7 +68464,7 @@
         <v>75</v>
       </c>
       <c r="G1674" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1674" s="10" t="s">
         <v>1789</v>
@@ -68476,7 +68473,7 @@
         <v>534</v>
       </c>
       <c r="J1674" s="7" t="s">
-        <v>2513</v>
+        <v>2512</v>
       </c>
       <c r="K1674" s="10" t="s">
         <v>1793</v>
@@ -68484,10 +68481,10 @@
     </row>
     <row r="1675" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1675" s="30" t="s">
+        <v>2517</v>
+      </c>
+      <c r="B1675" s="7" t="s">
         <v>2518</v>
-      </c>
-      <c r="B1675" s="7" t="s">
-        <v>2519</v>
       </c>
       <c r="C1675" s="7" t="s">
         <v>21</v>
@@ -68503,7 +68500,7 @@
         <v>35</v>
       </c>
       <c r="G1675" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1675" s="10" t="s">
         <v>1789</v>
@@ -68512,7 +68509,7 @@
         <v>534</v>
       </c>
       <c r="J1675" s="7" t="s">
-        <v>2513</v>
+        <v>2512</v>
       </c>
       <c r="K1675" s="10" t="s">
         <v>1793</v>
@@ -68520,10 +68517,10 @@
     </row>
     <row r="1676" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1676" s="30" t="s">
+        <v>2519</v>
+      </c>
+      <c r="B1676" s="7" t="s">
         <v>2520</v>
-      </c>
-      <c r="B1676" s="7" t="s">
-        <v>2521</v>
       </c>
       <c r="C1676" s="7" t="s">
         <v>21</v>
@@ -68539,7 +68536,7 @@
         <v>300</v>
       </c>
       <c r="G1676" s="7" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="H1676" s="10" t="s">
         <v>1789</v>
@@ -68548,7 +68545,7 @@
         <v>534</v>
       </c>
       <c r="J1676" s="7" t="s">
-        <v>2513</v>
+        <v>2512</v>
       </c>
       <c r="K1676" s="10" t="s">
         <v>1793</v>
@@ -68559,7 +68556,7 @@
         <v>216</v>
       </c>
       <c r="B1677" s="7" t="s">
-        <v>2522</v>
+        <v>2521</v>
       </c>
       <c r="C1677" s="7" t="s">
         <v>21</v>
@@ -68575,19 +68572,19 @@
         <v>400</v>
       </c>
       <c r="G1677" s="7" t="s">
+        <v>2522</v>
+      </c>
+      <c r="H1677" s="10" t="s">
         <v>2523</v>
-      </c>
-      <c r="H1677" s="10" t="s">
-        <v>2524</v>
       </c>
       <c r="I1677" s="7" t="s">
         <v>129</v>
       </c>
       <c r="J1677" s="7" t="s">
+        <v>2524</v>
+      </c>
+      <c r="K1677" s="10" t="s">
         <v>2525</v>
-      </c>
-      <c r="K1677" s="10" t="s">
-        <v>2526</v>
       </c>
     </row>
     <row r="1678" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -68595,7 +68592,7 @@
         <v>806</v>
       </c>
       <c r="B1678" s="7" t="s">
-        <v>2527</v>
+        <v>2526</v>
       </c>
       <c r="C1678" s="7" t="s">
         <v>62</v>
@@ -68611,27 +68608,27 @@
         <v>22610</v>
       </c>
       <c r="G1678" s="7" t="s">
-        <v>2528</v>
+        <v>2527</v>
       </c>
       <c r="H1678" s="10" t="s">
-        <v>2524</v>
+        <v>2523</v>
       </c>
       <c r="I1678" s="7" t="s">
         <v>77</v>
       </c>
       <c r="J1678" s="7" t="s">
-        <v>2529</v>
+        <v>2528</v>
       </c>
       <c r="K1678" s="10" t="s">
-        <v>2526</v>
+        <v>2525</v>
       </c>
     </row>
     <row r="1679" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1679" s="30" t="s">
+        <v>2529</v>
+      </c>
+      <c r="B1679" s="7" t="s">
         <v>2530</v>
-      </c>
-      <c r="B1679" s="7" t="s">
-        <v>2531</v>
       </c>
       <c r="C1679" s="7" t="s">
         <v>62</v>
@@ -68647,27 +68644,27 @@
         <v>14200</v>
       </c>
       <c r="G1679" s="7" t="s">
-        <v>2528</v>
+        <v>2527</v>
       </c>
       <c r="H1679" s="10" t="s">
-        <v>2524</v>
+        <v>2523</v>
       </c>
       <c r="I1679" s="7" t="s">
         <v>77</v>
       </c>
       <c r="J1679" s="7" t="s">
-        <v>2529</v>
+        <v>2528</v>
       </c>
       <c r="K1679" s="10" t="s">
-        <v>2526</v>
+        <v>2525</v>
       </c>
     </row>
     <row r="1680" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1680" s="30" t="s">
+        <v>2531</v>
+      </c>
+      <c r="B1680" s="7" t="s">
         <v>2532</v>
-      </c>
-      <c r="B1680" s="7" t="s">
-        <v>2533</v>
       </c>
       <c r="C1680" s="7" t="s">
         <v>21</v>
@@ -68683,19 +68680,19 @@
         <v>20000</v>
       </c>
       <c r="G1680" s="7" t="s">
+        <v>2533</v>
+      </c>
+      <c r="H1680" s="10" t="s">
         <v>2534</v>
-      </c>
-      <c r="H1680" s="10" t="s">
-        <v>2535</v>
       </c>
       <c r="I1680" s="7" t="s">
         <v>57</v>
       </c>
       <c r="J1680" s="7" t="s">
-        <v>2536</v>
+        <v>2535</v>
       </c>
       <c r="K1680" s="10" t="s">
-        <v>2526</v>
+        <v>2525</v>
       </c>
     </row>
     <row r="1681" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -68703,7 +68700,7 @@
         <v>577</v>
       </c>
       <c r="B1681" s="7" t="s">
-        <v>2537</v>
+        <v>2536</v>
       </c>
       <c r="C1681" s="7" t="s">
         <v>62</v>
@@ -68719,19 +68716,19 @@
         <v>8420.7999999999993</v>
       </c>
       <c r="G1681" s="7" t="s">
+        <v>2533</v>
+      </c>
+      <c r="H1681" s="10" t="s">
         <v>2534</v>
-      </c>
-      <c r="H1681" s="10" t="s">
-        <v>2535</v>
       </c>
       <c r="I1681" s="7" t="s">
         <v>57</v>
       </c>
       <c r="J1681" s="7" t="s">
-        <v>2536</v>
+        <v>2535</v>
       </c>
       <c r="K1681" s="10" t="s">
-        <v>2526</v>
+        <v>2525</v>
       </c>
     </row>
     <row r="1682" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -68739,7 +68736,7 @@
         <v>699</v>
       </c>
       <c r="B1682" s="7" t="s">
-        <v>2538</v>
+        <v>2537</v>
       </c>
       <c r="C1682" s="7" t="s">
         <v>62</v>
@@ -68755,19 +68752,19 @@
         <v>15788.999999999998</v>
       </c>
       <c r="G1682" s="7" t="s">
+        <v>2533</v>
+      </c>
+      <c r="H1682" s="10" t="s">
         <v>2534</v>
-      </c>
-      <c r="H1682" s="10" t="s">
-        <v>2535</v>
       </c>
       <c r="I1682" s="7" t="s">
         <v>57</v>
       </c>
       <c r="J1682" s="7" t="s">
-        <v>2536</v>
+        <v>2535</v>
       </c>
       <c r="K1682" s="10" t="s">
-        <v>2526</v>
+        <v>2525</v>
       </c>
     </row>
     <row r="1683" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -68775,7 +68772,7 @@
         <v>157</v>
       </c>
       <c r="B1683" s="10" t="s">
-        <v>2539</v>
+        <v>2538</v>
       </c>
       <c r="C1683" s="7" t="s">
         <v>21</v>
@@ -68791,7 +68788,7 @@
         <v>5557.5</v>
       </c>
       <c r="G1683" s="7" t="s">
-        <v>2540</v>
+        <v>2539</v>
       </c>
       <c r="H1683" s="10" t="s">
         <v>2332</v>
@@ -68800,7 +68797,7 @@
         <v>144</v>
       </c>
       <c r="J1683" s="7" t="s">
-        <v>2541</v>
+        <v>2540</v>
       </c>
       <c r="K1683" s="10">
         <v>46363</v>
@@ -68808,10 +68805,10 @@
     </row>
     <row r="1684" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1684" s="30" t="s">
+        <v>2541</v>
+      </c>
+      <c r="B1684" s="10" t="s">
         <v>2542</v>
-      </c>
-      <c r="B1684" s="10" t="s">
-        <v>2543</v>
       </c>
       <c r="C1684" s="7" t="s">
         <v>21</v>
@@ -68827,7 +68824,7 @@
         <v>1054</v>
       </c>
       <c r="G1684" s="7" t="s">
-        <v>2540</v>
+        <v>2539</v>
       </c>
       <c r="H1684" s="10" t="s">
         <v>2332</v>
@@ -68836,7 +68833,7 @@
         <v>144</v>
       </c>
       <c r="J1684" s="7" t="s">
-        <v>2541</v>
+        <v>2540</v>
       </c>
       <c r="K1684" s="10">
         <v>46363</v>
@@ -68844,10 +68841,10 @@
     </row>
     <row r="1685" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1685" s="30" t="s">
+        <v>2543</v>
+      </c>
+      <c r="B1685" s="10" t="s">
         <v>2544</v>
-      </c>
-      <c r="B1685" s="10" t="s">
-        <v>2545</v>
       </c>
       <c r="C1685" s="7" t="s">
         <v>21</v>
@@ -68863,7 +68860,7 @@
         <v>1266.99</v>
       </c>
       <c r="G1685" s="7" t="s">
-        <v>2540</v>
+        <v>2539</v>
       </c>
       <c r="H1685" s="10" t="s">
         <v>2332</v>
@@ -68872,7 +68869,7 @@
         <v>144</v>
       </c>
       <c r="J1685" s="7" t="s">
-        <v>2541</v>
+        <v>2540</v>
       </c>
       <c r="K1685" s="10">
         <v>46363</v>
@@ -68880,10 +68877,10 @@
     </row>
     <row r="1686" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1686" s="30" t="s">
+        <v>2545</v>
+      </c>
+      <c r="B1686" s="10" t="s">
         <v>2546</v>
-      </c>
-      <c r="B1686" s="10" t="s">
-        <v>2547</v>
       </c>
       <c r="C1686" s="7" t="s">
         <v>21</v>
@@ -68899,7 +68896,7 @@
         <v>9284</v>
       </c>
       <c r="G1686" s="7" t="s">
-        <v>2540</v>
+        <v>2539</v>
       </c>
       <c r="H1686" s="10" t="s">
         <v>2332</v>
@@ -68908,7 +68905,7 @@
         <v>144</v>
       </c>
       <c r="J1686" s="7" t="s">
-        <v>2541</v>
+        <v>2540</v>
       </c>
       <c r="K1686" s="10">
         <v>46363</v>
@@ -68916,10 +68913,10 @@
     </row>
     <row r="1687" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1687" s="30" t="s">
+        <v>2547</v>
+      </c>
+      <c r="B1687" s="10" t="s">
         <v>2548</v>
-      </c>
-      <c r="B1687" s="10" t="s">
-        <v>2549</v>
       </c>
       <c r="C1687" s="7" t="s">
         <v>21</v>
@@ -68935,7 +68932,7 @@
         <v>292.5</v>
       </c>
       <c r="G1687" s="7" t="s">
-        <v>2540</v>
+        <v>2539</v>
       </c>
       <c r="H1687" s="10" t="s">
         <v>2332</v>
@@ -68944,7 +68941,7 @@
         <v>144</v>
       </c>
       <c r="J1687" s="7" t="s">
-        <v>2541</v>
+        <v>2540</v>
       </c>
       <c r="K1687" s="10">
         <v>46363</v>
@@ -68952,10 +68949,10 @@
     </row>
     <row r="1688" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1688" s="30" t="s">
+        <v>2549</v>
+      </c>
+      <c r="B1688" s="10" t="s">
         <v>2550</v>
-      </c>
-      <c r="B1688" s="10" t="s">
-        <v>2551</v>
       </c>
       <c r="C1688" s="7" t="s">
         <v>21</v>
@@ -68971,7 +68968,7 @@
         <v>1930.5</v>
       </c>
       <c r="G1688" s="7" t="s">
-        <v>2540</v>
+        <v>2539</v>
       </c>
       <c r="H1688" s="10" t="s">
         <v>2332</v>
@@ -68980,7 +68977,7 @@
         <v>144</v>
       </c>
       <c r="J1688" s="7" t="s">
-        <v>2541</v>
+        <v>2540</v>
       </c>
       <c r="K1688" s="10">
         <v>46363</v>
@@ -68991,7 +68988,7 @@
         <v>904</v>
       </c>
       <c r="B1689" s="10" t="s">
-        <v>2552</v>
+        <v>2551</v>
       </c>
       <c r="C1689" s="7" t="s">
         <v>21</v>
@@ -69007,7 +69004,7 @@
         <v>3071.25</v>
       </c>
       <c r="G1689" s="7" t="s">
-        <v>2540</v>
+        <v>2539</v>
       </c>
       <c r="H1689" s="10" t="s">
         <v>2332</v>
@@ -69016,7 +69013,7 @@
         <v>144</v>
       </c>
       <c r="J1689" s="7" t="s">
-        <v>2541</v>
+        <v>2540</v>
       </c>
       <c r="K1689" s="10">
         <v>46363</v>
@@ -69024,10 +69021,10 @@
     </row>
     <row r="1690" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1690" s="30" t="s">
+        <v>2552</v>
+      </c>
+      <c r="B1690" s="10" t="s">
         <v>2553</v>
-      </c>
-      <c r="B1690" s="10" t="s">
-        <v>2554</v>
       </c>
       <c r="C1690" s="7" t="s">
         <v>21</v>
@@ -69043,7 +69040,7 @@
         <v>175.5</v>
       </c>
       <c r="G1690" s="7" t="s">
-        <v>2540</v>
+        <v>2539</v>
       </c>
       <c r="H1690" s="10" t="s">
         <v>2332</v>
@@ -69052,7 +69049,7 @@
         <v>144</v>
       </c>
       <c r="J1690" s="7" t="s">
-        <v>2541</v>
+        <v>2540</v>
       </c>
       <c r="K1690" s="10">
         <v>46363</v>
@@ -69063,7 +69060,7 @@
         <v>201</v>
       </c>
       <c r="B1691" s="10" t="s">
-        <v>2555</v>
+        <v>2554</v>
       </c>
       <c r="C1691" s="10" t="s">
         <v>21</v>
@@ -69079,16 +69076,16 @@
         <v>2750</v>
       </c>
       <c r="G1691" s="7" t="s">
+        <v>2555</v>
+      </c>
+      <c r="H1691" s="10" t="s">
         <v>2556</v>
-      </c>
-      <c r="H1691" s="10" t="s">
-        <v>2557</v>
       </c>
       <c r="I1691" s="7" t="s">
         <v>203</v>
       </c>
       <c r="J1691" s="10" t="s">
-        <v>2558</v>
+        <v>2557</v>
       </c>
       <c r="K1691" s="10">
         <v>46363</v>
@@ -69099,7 +69096,7 @@
         <v>205</v>
       </c>
       <c r="B1692" s="10" t="s">
-        <v>2559</v>
+        <v>2558</v>
       </c>
       <c r="C1692" s="10" t="s">
         <v>21</v>
@@ -69115,16 +69112,16 @@
         <v>750</v>
       </c>
       <c r="G1692" s="7" t="s">
+        <v>2555</v>
+      </c>
+      <c r="H1692" s="10" t="s">
         <v>2556</v>
-      </c>
-      <c r="H1692" s="10" t="s">
-        <v>2557</v>
       </c>
       <c r="I1692" s="7" t="s">
         <v>203</v>
       </c>
       <c r="J1692" s="10" t="s">
-        <v>2558</v>
+        <v>2557</v>
       </c>
       <c r="K1692" s="10">
         <v>46363</v>
@@ -69135,7 +69132,7 @@
         <v>297</v>
       </c>
       <c r="B1693" s="10" t="s">
-        <v>2560</v>
+        <v>2559</v>
       </c>
       <c r="C1693" s="10" t="s">
         <v>21</v>
@@ -69151,16 +69148,16 @@
         <v>3200</v>
       </c>
       <c r="G1693" s="7" t="s">
+        <v>2555</v>
+      </c>
+      <c r="H1693" s="10" t="s">
         <v>2556</v>
-      </c>
-      <c r="H1693" s="10" t="s">
-        <v>2557</v>
       </c>
       <c r="I1693" s="7" t="s">
         <v>203</v>
       </c>
       <c r="J1693" s="10" t="s">
-        <v>2558</v>
+        <v>2557</v>
       </c>
       <c r="K1693" s="10">
         <v>46363</v>
@@ -69171,7 +69168,7 @@
         <v>1528</v>
       </c>
       <c r="B1694" s="7" t="s">
-        <v>2561</v>
+        <v>2560</v>
       </c>
       <c r="C1694" s="10" t="s">
         <v>21</v>
@@ -69187,27 +69184,27 @@
         <v>131614</v>
       </c>
       <c r="G1694" s="7" t="s">
+        <v>2561</v>
+      </c>
+      <c r="H1694" s="10" t="s">
+        <v>2556</v>
+      </c>
+      <c r="I1694" s="7" t="s">
         <v>2562</v>
       </c>
-      <c r="H1694" s="10" t="s">
-        <v>2557</v>
-      </c>
-      <c r="I1694" s="7" t="s">
+      <c r="J1694" s="7" t="s">
         <v>2563</v>
       </c>
-      <c r="J1694" s="7" t="s">
+      <c r="K1694" s="10" t="s">
         <v>2564</v>
-      </c>
-      <c r="K1694" s="10" t="s">
-        <v>2565</v>
       </c>
     </row>
     <row r="1695" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1695" s="30" t="s">
+        <v>2565</v>
+      </c>
+      <c r="B1695" s="7" t="s">
         <v>2566</v>
-      </c>
-      <c r="B1695" s="7" t="s">
-        <v>2567</v>
       </c>
       <c r="C1695" s="10" t="s">
         <v>21</v>
@@ -69223,27 +69220,27 @@
         <v>222882</v>
       </c>
       <c r="G1695" s="7" t="s">
+        <v>2561</v>
+      </c>
+      <c r="H1695" s="10" t="s">
+        <v>2556</v>
+      </c>
+      <c r="I1695" s="7" t="s">
         <v>2562</v>
       </c>
-      <c r="H1695" s="10" t="s">
-        <v>2557</v>
-      </c>
-      <c r="I1695" s="7" t="s">
+      <c r="J1695" s="7" t="s">
         <v>2563</v>
       </c>
-      <c r="J1695" s="7" t="s">
+      <c r="K1695" s="10" t="s">
         <v>2564</v>
-      </c>
-      <c r="K1695" s="10" t="s">
-        <v>2565</v>
       </c>
     </row>
     <row r="1696" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1696" s="6" t="s">
+        <v>2567</v>
+      </c>
+      <c r="B1696" s="7" t="s">
         <v>2568</v>
-      </c>
-      <c r="B1696" s="7" t="s">
-        <v>2569</v>
       </c>
       <c r="C1696" s="10" t="s">
         <v>21</v>
@@ -69259,7 +69256,7 @@
         <v>15684.300000000001</v>
       </c>
       <c r="G1696" s="7" t="s">
-        <v>2570</v>
+        <v>2569</v>
       </c>
       <c r="H1696" s="10">
         <v>46327</v>
@@ -69268,7 +69265,7 @@
         <v>804</v>
       </c>
       <c r="J1696" s="7" t="s">
-        <v>2571</v>
+        <v>2570</v>
       </c>
       <c r="K1696" s="10" t="s">
         <v>71</v>
@@ -69276,10 +69273,10 @@
     </row>
     <row r="1697" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1697" s="6" t="s">
+        <v>2571</v>
+      </c>
+      <c r="B1697" s="7" t="s">
         <v>2572</v>
-      </c>
-      <c r="B1697" s="7" t="s">
-        <v>2573</v>
       </c>
       <c r="C1697" s="10" t="s">
         <v>21</v>
@@ -69295,7 +69292,7 @@
         <v>4966.7900000000009</v>
       </c>
       <c r="G1697" s="7" t="s">
-        <v>2570</v>
+        <v>2569</v>
       </c>
       <c r="H1697" s="10">
         <v>46327</v>
@@ -69304,7 +69301,7 @@
         <v>804</v>
       </c>
       <c r="J1697" s="7" t="s">
-        <v>2571</v>
+        <v>2570</v>
       </c>
       <c r="K1697" s="10" t="s">
         <v>71</v>
@@ -69313,7 +69310,7 @@
     <row r="1698" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1698" s="6"/>
       <c r="B1698" s="7" t="s">
-        <v>2574</v>
+        <v>2573</v>
       </c>
       <c r="C1698" s="10" t="s">
         <v>21</v>
@@ -69329,7 +69326,7 @@
         <v>10054.800000000001</v>
       </c>
       <c r="G1698" s="7" t="s">
-        <v>2570</v>
+        <v>2569</v>
       </c>
       <c r="H1698" s="10">
         <v>46327</v>
@@ -69338,7 +69335,7 @@
         <v>804</v>
       </c>
       <c r="J1698" s="7" t="s">
-        <v>2571</v>
+        <v>2570</v>
       </c>
       <c r="K1698" s="10" t="s">
         <v>71</v>
@@ -69347,7 +69344,7 @@
     <row r="1699" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1699" s="6"/>
       <c r="B1699" s="7" t="s">
-        <v>2575</v>
+        <v>2574</v>
       </c>
       <c r="C1699" s="10" t="s">
         <v>21</v>
@@ -69363,7 +69360,7 @@
         <v>2280</v>
       </c>
       <c r="G1699" s="7" t="s">
-        <v>2570</v>
+        <v>2569</v>
       </c>
       <c r="H1699" s="10">
         <v>46327</v>
@@ -69372,7 +69369,7 @@
         <v>804</v>
       </c>
       <c r="J1699" s="7" t="s">
-        <v>2571</v>
+        <v>2570</v>
       </c>
       <c r="K1699" s="10" t="s">
         <v>71</v>

</xml_diff>

<commit_message>
Update all.xlsx file with the latest transaction data revisions
</commit_message>
<xml_diff>
--- a/data/transactions/all.xlsx
+++ b/data/transactions/all.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24332"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB866F8F-3AC0-47F0-B6CA-86F5AB4C425A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F21E2912-FC40-4F9D-B3F2-51BA1939BFD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9258" uniqueCount="2580">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9254" uniqueCount="2580">
   <si>
     <t>كود الصنف</t>
   </si>
@@ -8314,7 +8314,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P1700"/>
+  <dimension ref="A1:P1699"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.42578125" style="23" customWidth="1"/>
@@ -66134,7 +66134,7 @@
         <v>90.957490000000007</v>
       </c>
       <c r="F1609" s="9">
-        <f t="shared" ref="F1609:F1699" si="26">E1609*D1609</f>
+        <f t="shared" ref="F1609:F1698" si="26">E1609*D1609</f>
         <v>90957.49</v>
       </c>
       <c r="G1609" s="7">
@@ -66580,25 +66580,27 @@
       </c>
     </row>
     <row r="1622" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1622" s="30"/>
+      <c r="A1622" s="30" t="s">
+        <v>2422</v>
+      </c>
       <c r="B1622" s="7" t="s">
-        <v>1534</v>
+        <v>1535</v>
       </c>
       <c r="C1622" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1622" s="8">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E1622" s="8">
-        <v>15</v>
+        <v>190</v>
       </c>
       <c r="F1622" s="9">
         <f t="shared" si="26"/>
-        <v>450</v>
+        <v>950</v>
       </c>
       <c r="G1622" s="7">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="H1622" s="10">
         <v>46146</v>
@@ -66607,7 +66609,7 @@
         <v>54</v>
       </c>
       <c r="J1622" s="7">
-        <v>6303</v>
+        <v>6304</v>
       </c>
       <c r="K1622" s="10" t="s">
         <v>1501</v>
@@ -66615,59 +66617,59 @@
     </row>
     <row r="1623" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1623" s="30" t="s">
-        <v>2422</v>
+        <v>2423</v>
       </c>
       <c r="B1623" s="7" t="s">
-        <v>1535</v>
+        <v>2424</v>
       </c>
       <c r="C1623" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1623" s="8">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E1623" s="8">
-        <v>190</v>
+        <v>2015</v>
       </c>
       <c r="F1623" s="9">
         <f t="shared" si="26"/>
-        <v>950</v>
-      </c>
-      <c r="G1623" s="7">
-        <v>136</v>
-      </c>
-      <c r="H1623" s="10">
-        <v>46146</v>
+        <v>4030</v>
+      </c>
+      <c r="G1623" s="7" t="s">
+        <v>2425</v>
+      </c>
+      <c r="H1623" s="10" t="s">
+        <v>2426</v>
       </c>
       <c r="I1623" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="J1623" s="7">
-        <v>6304</v>
+        <v>2427</v>
+      </c>
+      <c r="J1623" s="7" t="s">
+        <v>2428</v>
       </c>
       <c r="K1623" s="10" t="s">
-        <v>1501</v>
+        <v>2429</v>
       </c>
     </row>
     <row r="1624" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1624" s="30" t="s">
-        <v>2423</v>
+        <v>2430</v>
       </c>
       <c r="B1624" s="7" t="s">
-        <v>2424</v>
+        <v>2431</v>
       </c>
       <c r="C1624" s="7" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="D1624" s="8">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E1624" s="8">
-        <v>2015</v>
+        <v>1400</v>
       </c>
       <c r="F1624" s="9">
         <f t="shared" si="26"/>
-        <v>4030</v>
+        <v>7000</v>
       </c>
       <c r="G1624" s="7" t="s">
         <v>2425</v>
@@ -66687,59 +66689,59 @@
     </row>
     <row r="1625" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1625" s="30" t="s">
-        <v>2430</v>
+        <v>609</v>
       </c>
       <c r="B1625" s="7" t="s">
-        <v>2431</v>
+        <v>2432</v>
       </c>
       <c r="C1625" s="7" t="s">
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="D1625" s="8">
-        <v>5</v>
+        <v>300</v>
       </c>
       <c r="E1625" s="8">
-        <v>1400</v>
+        <v>2021.05</v>
       </c>
       <c r="F1625" s="9">
         <f t="shared" si="26"/>
-        <v>7000</v>
+        <v>606315</v>
       </c>
       <c r="G1625" s="7" t="s">
-        <v>2425</v>
+        <v>2433</v>
       </c>
       <c r="H1625" s="10" t="s">
-        <v>2426</v>
+        <v>1783</v>
       </c>
       <c r="I1625" s="7" t="s">
-        <v>2427</v>
+        <v>2434</v>
       </c>
       <c r="J1625" s="7" t="s">
-        <v>2428</v>
+        <v>2435</v>
       </c>
       <c r="K1625" s="10" t="s">
-        <v>2429</v>
+        <v>2436</v>
       </c>
     </row>
     <row r="1626" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1626" s="30" t="s">
-        <v>609</v>
+        <v>1737</v>
       </c>
       <c r="B1626" s="7" t="s">
-        <v>2432</v>
+        <v>2437</v>
       </c>
       <c r="C1626" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1626" s="8">
-        <v>300</v>
+        <v>72</v>
       </c>
       <c r="E1626" s="8">
-        <v>2021.05</v>
+        <v>3157.89</v>
       </c>
       <c r="F1626" s="9">
         <f t="shared" si="26"/>
-        <v>606315</v>
+        <v>227368.08</v>
       </c>
       <c r="G1626" s="7" t="s">
         <v>2433</v>
@@ -66759,23 +66761,23 @@
     </row>
     <row r="1627" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1627" s="30" t="s">
-        <v>1737</v>
+        <v>577</v>
       </c>
       <c r="B1627" s="7" t="s">
-        <v>2437</v>
+        <v>2438</v>
       </c>
       <c r="C1627" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1627" s="8">
-        <v>72</v>
+        <v>29</v>
       </c>
       <c r="E1627" s="8">
-        <v>3157.89</v>
+        <v>4736.8900000000003</v>
       </c>
       <c r="F1627" s="9">
         <f t="shared" si="26"/>
-        <v>227368.08</v>
+        <v>137369.81</v>
       </c>
       <c r="G1627" s="7" t="s">
         <v>2433</v>
@@ -66795,46 +66797,46 @@
     </row>
     <row r="1628" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1628" s="30" t="s">
-        <v>577</v>
+        <v>2439</v>
       </c>
       <c r="B1628" s="7" t="s">
-        <v>2438</v>
+        <v>2440</v>
       </c>
       <c r="C1628" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1628" s="8">
-        <v>29</v>
+        <v>50</v>
       </c>
       <c r="E1628" s="8">
-        <v>4736.8900000000003</v>
+        <v>75</v>
       </c>
       <c r="F1628" s="9">
         <f t="shared" si="26"/>
-        <v>137369.81</v>
+        <v>3750</v>
       </c>
       <c r="G1628" s="7" t="s">
-        <v>2433</v>
+        <v>2441</v>
       </c>
       <c r="H1628" s="10" t="s">
-        <v>1783</v>
+        <v>1789</v>
       </c>
       <c r="I1628" s="7" t="s">
-        <v>2434</v>
+        <v>534</v>
       </c>
       <c r="J1628" s="7" t="s">
-        <v>2435</v>
+        <v>2442</v>
       </c>
       <c r="K1628" s="10" t="s">
-        <v>2436</v>
+        <v>1793</v>
       </c>
     </row>
     <row r="1629" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1629" s="30" t="s">
-        <v>2439</v>
+        <v>2443</v>
       </c>
       <c r="B1629" s="7" t="s">
-        <v>2440</v>
+        <v>2444</v>
       </c>
       <c r="C1629" s="7" t="s">
         <v>21</v>
@@ -66843,11 +66845,11 @@
         <v>50</v>
       </c>
       <c r="E1629" s="8">
-        <v>75</v>
+        <v>375</v>
       </c>
       <c r="F1629" s="9">
         <f t="shared" si="26"/>
-        <v>3750</v>
+        <v>18750</v>
       </c>
       <c r="G1629" s="7" t="s">
         <v>2441</v>
@@ -66867,19 +66869,19 @@
     </row>
     <row r="1630" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1630" s="30" t="s">
-        <v>2443</v>
+        <v>892</v>
       </c>
       <c r="B1630" s="7" t="s">
-        <v>2444</v>
+        <v>893</v>
       </c>
       <c r="C1630" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1630" s="8">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="E1630" s="8">
-        <v>375</v>
+        <v>750</v>
       </c>
       <c r="F1630" s="9">
         <f t="shared" si="26"/>
@@ -66903,23 +66905,23 @@
     </row>
     <row r="1631" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1631" s="30" t="s">
-        <v>892</v>
+        <v>2445</v>
       </c>
       <c r="B1631" s="7" t="s">
-        <v>893</v>
+        <v>2446</v>
       </c>
       <c r="C1631" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1631" s="8">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="E1631" s="8">
-        <v>750</v>
+        <v>15</v>
       </c>
       <c r="F1631" s="9">
         <f t="shared" si="26"/>
-        <v>18750</v>
+        <v>300</v>
       </c>
       <c r="G1631" s="7" t="s">
         <v>2441</v>
@@ -66939,23 +66941,23 @@
     </row>
     <row r="1632" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1632" s="30" t="s">
-        <v>2445</v>
+        <v>2447</v>
       </c>
       <c r="B1632" s="7" t="s">
-        <v>2446</v>
+        <v>2448</v>
       </c>
       <c r="C1632" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1632" s="8">
+        <v>10</v>
+      </c>
+      <c r="E1632" s="8">
         <v>20</v>
-      </c>
-      <c r="E1632" s="8">
-        <v>15</v>
       </c>
       <c r="F1632" s="9">
         <f t="shared" si="26"/>
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="G1632" s="7" t="s">
         <v>2441</v>
@@ -66975,23 +66977,23 @@
     </row>
     <row r="1633" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1633" s="30" t="s">
-        <v>2447</v>
+        <v>2449</v>
       </c>
       <c r="B1633" s="7" t="s">
-        <v>2448</v>
+        <v>2450</v>
       </c>
       <c r="C1633" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1633" s="8">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E1633" s="8">
-        <v>20</v>
+        <v>675</v>
       </c>
       <c r="F1633" s="9">
         <f t="shared" si="26"/>
-        <v>200</v>
+        <v>3375</v>
       </c>
       <c r="G1633" s="7" t="s">
         <v>2441</v>
@@ -67011,23 +67013,23 @@
     </row>
     <row r="1634" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1634" s="30" t="s">
-        <v>2449</v>
+        <v>537</v>
       </c>
       <c r="B1634" s="7" t="s">
-        <v>2450</v>
+        <v>2451</v>
       </c>
       <c r="C1634" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1634" s="8">
-        <v>5</v>
+        <v>50</v>
       </c>
       <c r="E1634" s="8">
-        <v>675</v>
+        <v>15</v>
       </c>
       <c r="F1634" s="9">
         <f t="shared" si="26"/>
-        <v>3375</v>
+        <v>750</v>
       </c>
       <c r="G1634" s="7" t="s">
         <v>2441</v>
@@ -67047,23 +67049,23 @@
     </row>
     <row r="1635" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1635" s="30" t="s">
-        <v>537</v>
+        <v>2452</v>
       </c>
       <c r="B1635" s="7" t="s">
-        <v>2451</v>
+        <v>2453</v>
       </c>
       <c r="C1635" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1635" s="8">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="E1635" s="8">
         <v>15</v>
       </c>
       <c r="F1635" s="9">
         <f t="shared" si="26"/>
-        <v>750</v>
+        <v>1500</v>
       </c>
       <c r="G1635" s="7" t="s">
         <v>2441</v>
@@ -67083,10 +67085,10 @@
     </row>
     <row r="1636" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1636" s="30" t="s">
-        <v>2452</v>
+        <v>2454</v>
       </c>
       <c r="B1636" s="7" t="s">
-        <v>2453</v>
+        <v>2455</v>
       </c>
       <c r="C1636" s="7" t="s">
         <v>21</v>
@@ -67095,11 +67097,11 @@
         <v>100</v>
       </c>
       <c r="E1636" s="8">
-        <v>15</v>
+        <v>48</v>
       </c>
       <c r="F1636" s="9">
         <f t="shared" si="26"/>
-        <v>1500</v>
+        <v>4800</v>
       </c>
       <c r="G1636" s="7" t="s">
         <v>2441</v>
@@ -67119,23 +67121,23 @@
     </row>
     <row r="1637" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1637" s="30" t="s">
-        <v>2454</v>
+        <v>539</v>
       </c>
       <c r="B1637" s="7" t="s">
-        <v>2455</v>
+        <v>540</v>
       </c>
       <c r="C1637" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1637" s="8">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="E1637" s="8">
-        <v>48</v>
+        <v>25</v>
       </c>
       <c r="F1637" s="9">
         <f t="shared" si="26"/>
-        <v>4800</v>
+        <v>1250</v>
       </c>
       <c r="G1637" s="7" t="s">
         <v>2441</v>
@@ -67155,26 +67157,26 @@
     </row>
     <row r="1638" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1638" s="30" t="s">
-        <v>539</v>
+        <v>847</v>
       </c>
       <c r="B1638" s="7" t="s">
-        <v>540</v>
+        <v>2456</v>
       </c>
       <c r="C1638" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1638" s="8">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="E1638" s="8">
-        <v>25</v>
+        <v>125</v>
       </c>
       <c r="F1638" s="9">
         <f t="shared" si="26"/>
-        <v>1250</v>
+        <v>5625</v>
       </c>
       <c r="G1638" s="7" t="s">
-        <v>2441</v>
+        <v>2457</v>
       </c>
       <c r="H1638" s="10" t="s">
         <v>1789</v>
@@ -67183,7 +67185,7 @@
         <v>534</v>
       </c>
       <c r="J1638" s="7" t="s">
-        <v>2442</v>
+        <v>2458</v>
       </c>
       <c r="K1638" s="10" t="s">
         <v>1793</v>
@@ -67191,23 +67193,23 @@
     </row>
     <row r="1639" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1639" s="30" t="s">
-        <v>847</v>
+        <v>2459</v>
       </c>
       <c r="B1639" s="7" t="s">
-        <v>2456</v>
+        <v>2460</v>
       </c>
       <c r="C1639" s="7" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="D1639" s="8">
-        <v>45</v>
+        <v>5</v>
       </c>
       <c r="E1639" s="8">
-        <v>125</v>
+        <v>450</v>
       </c>
       <c r="F1639" s="9">
         <f t="shared" si="26"/>
-        <v>5625</v>
+        <v>2250</v>
       </c>
       <c r="G1639" s="7" t="s">
         <v>2457</v>
@@ -67227,19 +67229,19 @@
     </row>
     <row r="1640" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1640" s="30" t="s">
-        <v>2459</v>
+        <v>2461</v>
       </c>
       <c r="B1640" s="7" t="s">
-        <v>2460</v>
+        <v>2462</v>
       </c>
       <c r="C1640" s="7" t="s">
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="D1640" s="8">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E1640" s="8">
-        <v>450</v>
+        <v>2250</v>
       </c>
       <c r="F1640" s="9">
         <f t="shared" si="26"/>
@@ -67263,10 +67265,10 @@
     </row>
     <row r="1641" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1641" s="30" t="s">
-        <v>2461</v>
+        <v>2463</v>
       </c>
       <c r="B1641" s="7" t="s">
-        <v>2462</v>
+        <v>2464</v>
       </c>
       <c r="C1641" s="7" t="s">
         <v>21</v>
@@ -67275,11 +67277,11 @@
         <v>1</v>
       </c>
       <c r="E1641" s="8">
-        <v>2250</v>
+        <v>575</v>
       </c>
       <c r="F1641" s="9">
         <f t="shared" si="26"/>
-        <v>2250</v>
+        <v>575</v>
       </c>
       <c r="G1641" s="7" t="s">
         <v>2457</v>
@@ -67299,23 +67301,23 @@
     </row>
     <row r="1642" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1642" s="30" t="s">
-        <v>2463</v>
+        <v>2465</v>
       </c>
       <c r="B1642" s="7" t="s">
-        <v>2464</v>
+        <v>2065</v>
       </c>
       <c r="C1642" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1642" s="8">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E1642" s="8">
-        <v>575</v>
+        <v>125</v>
       </c>
       <c r="F1642" s="9">
         <f t="shared" si="26"/>
-        <v>575</v>
+        <v>500</v>
       </c>
       <c r="G1642" s="7" t="s">
         <v>2457</v>
@@ -67335,23 +67337,23 @@
     </row>
     <row r="1643" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1643" s="30" t="s">
-        <v>2465</v>
+        <v>2452</v>
       </c>
       <c r="B1643" s="7" t="s">
-        <v>2065</v>
+        <v>2453</v>
       </c>
       <c r="C1643" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1643" s="8">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E1643" s="8">
-        <v>125</v>
+        <v>15</v>
       </c>
       <c r="F1643" s="9">
         <f t="shared" si="26"/>
-        <v>500</v>
+        <v>90</v>
       </c>
       <c r="G1643" s="7" t="s">
         <v>2457</v>
@@ -67371,23 +67373,23 @@
     </row>
     <row r="1644" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1644" s="30" t="s">
-        <v>2452</v>
+        <v>2466</v>
       </c>
       <c r="B1644" s="7" t="s">
-        <v>2453</v>
+        <v>2467</v>
       </c>
       <c r="C1644" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1644" s="8">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E1644" s="8">
-        <v>15</v>
+        <v>75</v>
       </c>
       <c r="F1644" s="9">
         <f t="shared" si="26"/>
-        <v>90</v>
+        <v>675</v>
       </c>
       <c r="G1644" s="7" t="s">
         <v>2457</v>
@@ -67407,23 +67409,23 @@
     </row>
     <row r="1645" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1645" s="30" t="s">
-        <v>2466</v>
+        <v>2468</v>
       </c>
       <c r="B1645" s="7" t="s">
-        <v>2467</v>
+        <v>2469</v>
       </c>
       <c r="C1645" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1645" s="8">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E1645" s="8">
-        <v>75</v>
+        <v>2750</v>
       </c>
       <c r="F1645" s="9">
         <f t="shared" si="26"/>
-        <v>675</v>
+        <v>11000</v>
       </c>
       <c r="G1645" s="7" t="s">
         <v>2457</v>
@@ -67443,10 +67445,10 @@
     </row>
     <row r="1646" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1646" s="30" t="s">
-        <v>2468</v>
+        <v>535</v>
       </c>
       <c r="B1646" s="7" t="s">
-        <v>2469</v>
+        <v>2470</v>
       </c>
       <c r="C1646" s="7" t="s">
         <v>21</v>
@@ -67455,11 +67457,11 @@
         <v>4</v>
       </c>
       <c r="E1646" s="8">
-        <v>2750</v>
+        <v>75</v>
       </c>
       <c r="F1646" s="9">
         <f t="shared" si="26"/>
-        <v>11000</v>
+        <v>300</v>
       </c>
       <c r="G1646" s="7" t="s">
         <v>2457</v>
@@ -67479,10 +67481,10 @@
     </row>
     <row r="1647" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1647" s="30" t="s">
-        <v>535</v>
+        <v>2471</v>
       </c>
       <c r="B1647" s="7" t="s">
-        <v>2470</v>
+        <v>2472</v>
       </c>
       <c r="C1647" s="7" t="s">
         <v>21</v>
@@ -67515,23 +67517,23 @@
     </row>
     <row r="1648" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1648" s="30" t="s">
-        <v>2471</v>
+        <v>2473</v>
       </c>
       <c r="B1648" s="7" t="s">
-        <v>2472</v>
+        <v>2474</v>
       </c>
       <c r="C1648" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1648" s="8">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E1648" s="8">
         <v>75</v>
       </c>
       <c r="F1648" s="9">
         <f t="shared" si="26"/>
-        <v>300</v>
+        <v>150</v>
       </c>
       <c r="G1648" s="7" t="s">
         <v>2457</v>
@@ -67551,23 +67553,23 @@
     </row>
     <row r="1649" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1649" s="30" t="s">
-        <v>2473</v>
+        <v>2475</v>
       </c>
       <c r="B1649" s="7" t="s">
-        <v>2474</v>
+        <v>2476</v>
       </c>
       <c r="C1649" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1649" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E1649" s="8">
-        <v>75</v>
+        <v>275</v>
       </c>
       <c r="F1649" s="9">
         <f t="shared" si="26"/>
-        <v>150</v>
+        <v>275</v>
       </c>
       <c r="G1649" s="7" t="s">
         <v>2457</v>
@@ -67579,7 +67581,7 @@
         <v>534</v>
       </c>
       <c r="J1649" s="7" t="s">
-        <v>2458</v>
+        <v>2477</v>
       </c>
       <c r="K1649" s="10" t="s">
         <v>1793</v>
@@ -67587,10 +67589,10 @@
     </row>
     <row r="1650" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1650" s="30" t="s">
-        <v>2475</v>
+        <v>2478</v>
       </c>
       <c r="B1650" s="7" t="s">
-        <v>2476</v>
+        <v>2479</v>
       </c>
       <c r="C1650" s="7" t="s">
         <v>21</v>
@@ -67599,11 +67601,11 @@
         <v>1</v>
       </c>
       <c r="E1650" s="8">
-        <v>275</v>
+        <v>3000</v>
       </c>
       <c r="F1650" s="9">
         <f t="shared" si="26"/>
-        <v>275</v>
+        <v>3000</v>
       </c>
       <c r="G1650" s="7" t="s">
         <v>2457</v>
@@ -67623,23 +67625,23 @@
     </row>
     <row r="1651" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1651" s="30" t="s">
-        <v>2478</v>
+        <v>2577</v>
       </c>
       <c r="B1651" s="7" t="s">
-        <v>2479</v>
+        <v>2481</v>
       </c>
       <c r="C1651" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1651" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E1651" s="8">
-        <v>3000</v>
+        <v>750</v>
       </c>
       <c r="F1651" s="9">
         <f t="shared" si="26"/>
-        <v>3000</v>
+        <v>1500</v>
       </c>
       <c r="G1651" s="7" t="s">
         <v>2457</v>
@@ -67659,23 +67661,23 @@
     </row>
     <row r="1652" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1652" s="30" t="s">
-        <v>2577</v>
+        <v>2482</v>
       </c>
       <c r="B1652" s="7" t="s">
-        <v>2481</v>
+        <v>2483</v>
       </c>
       <c r="C1652" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1652" s="8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E1652" s="8">
-        <v>750</v>
+        <v>25</v>
       </c>
       <c r="F1652" s="9">
         <f t="shared" si="26"/>
-        <v>1500</v>
+        <v>100</v>
       </c>
       <c r="G1652" s="7" t="s">
         <v>2457</v>
@@ -67695,23 +67697,23 @@
     </row>
     <row r="1653" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1653" s="30" t="s">
-        <v>2482</v>
+        <v>2484</v>
       </c>
       <c r="B1653" s="7" t="s">
-        <v>2483</v>
+        <v>2485</v>
       </c>
       <c r="C1653" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1653" s="8">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E1653" s="8">
-        <v>25</v>
+        <v>75</v>
       </c>
       <c r="F1653" s="9">
         <f t="shared" si="26"/>
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="G1653" s="7" t="s">
         <v>2457</v>
@@ -67731,23 +67733,23 @@
     </row>
     <row r="1654" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1654" s="30" t="s">
-        <v>2484</v>
+        <v>2486</v>
       </c>
       <c r="B1654" s="7" t="s">
-        <v>2485</v>
+        <v>2487</v>
       </c>
       <c r="C1654" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1654" s="8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E1654" s="8">
-        <v>75</v>
+        <v>185</v>
       </c>
       <c r="F1654" s="9">
         <f t="shared" si="26"/>
-        <v>75</v>
+        <v>925</v>
       </c>
       <c r="G1654" s="7" t="s">
         <v>2457</v>
@@ -67767,10 +67769,10 @@
     </row>
     <row r="1655" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1655" s="30" t="s">
-        <v>2486</v>
+        <v>2488</v>
       </c>
       <c r="B1655" s="7" t="s">
-        <v>2487</v>
+        <v>2489</v>
       </c>
       <c r="C1655" s="7" t="s">
         <v>21</v>
@@ -67779,11 +67781,11 @@
         <v>5</v>
       </c>
       <c r="E1655" s="8">
-        <v>185</v>
+        <v>3450</v>
       </c>
       <c r="F1655" s="9">
         <f t="shared" si="26"/>
-        <v>925</v>
+        <v>17250</v>
       </c>
       <c r="G1655" s="7" t="s">
         <v>2457</v>
@@ -67803,10 +67805,10 @@
     </row>
     <row r="1656" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1656" s="30" t="s">
-        <v>2488</v>
+        <v>2490</v>
       </c>
       <c r="B1656" s="7" t="s">
-        <v>2489</v>
+        <v>2491</v>
       </c>
       <c r="C1656" s="7" t="s">
         <v>21</v>
@@ -67815,11 +67817,11 @@
         <v>5</v>
       </c>
       <c r="E1656" s="8">
-        <v>3450</v>
+        <v>450</v>
       </c>
       <c r="F1656" s="9">
         <f t="shared" si="26"/>
-        <v>17250</v>
+        <v>2250</v>
       </c>
       <c r="G1656" s="7" t="s">
         <v>2457</v>
@@ -67839,23 +67841,23 @@
     </row>
     <row r="1657" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1657" s="30" t="s">
-        <v>2490</v>
+        <v>841</v>
       </c>
       <c r="B1657" s="7" t="s">
-        <v>2491</v>
+        <v>2492</v>
       </c>
       <c r="C1657" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1657" s="8">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E1657" s="8">
-        <v>450</v>
+        <v>35</v>
       </c>
       <c r="F1657" s="9">
         <f t="shared" si="26"/>
-        <v>2250</v>
+        <v>70</v>
       </c>
       <c r="G1657" s="7" t="s">
         <v>2457</v>
@@ -67875,23 +67877,23 @@
     </row>
     <row r="1658" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1658" s="30" t="s">
-        <v>841</v>
+        <v>2067</v>
       </c>
       <c r="B1658" s="7" t="s">
-        <v>2492</v>
+        <v>2493</v>
       </c>
       <c r="C1658" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1658" s="8">
-        <v>2</v>
+        <v>35</v>
       </c>
       <c r="E1658" s="8">
         <v>35</v>
       </c>
       <c r="F1658" s="9">
         <f t="shared" si="26"/>
-        <v>70</v>
+        <v>1225</v>
       </c>
       <c r="G1658" s="7" t="s">
         <v>2457</v>
@@ -67911,23 +67913,23 @@
     </row>
     <row r="1659" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1659" s="30" t="s">
-        <v>2067</v>
+        <v>2578</v>
       </c>
       <c r="B1659" s="7" t="s">
-        <v>2493</v>
+        <v>2495</v>
       </c>
       <c r="C1659" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1659" s="8">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="E1659" s="8">
-        <v>35</v>
+        <v>175</v>
       </c>
       <c r="F1659" s="9">
         <f t="shared" si="26"/>
-        <v>1225</v>
+        <v>1750</v>
       </c>
       <c r="G1659" s="7" t="s">
         <v>2457</v>
@@ -67946,24 +67948,22 @@
       </c>
     </row>
     <row r="1660" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1660" s="30" t="s">
-        <v>2578</v>
-      </c>
+      <c r="A1660" s="6"/>
       <c r="B1660" s="7" t="s">
-        <v>2495</v>
+        <v>2496</v>
       </c>
       <c r="C1660" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1660" s="8">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="E1660" s="8">
-        <v>175</v>
+        <v>28</v>
       </c>
       <c r="F1660" s="9">
         <f t="shared" si="26"/>
-        <v>1750</v>
+        <v>1540</v>
       </c>
       <c r="G1660" s="7" t="s">
         <v>2457</v>
@@ -67975,7 +67975,7 @@
         <v>534</v>
       </c>
       <c r="J1660" s="7" t="s">
-        <v>2477</v>
+        <v>2497</v>
       </c>
       <c r="K1660" s="10" t="s">
         <v>1793</v>
@@ -67984,20 +67984,20 @@
     <row r="1661" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1661" s="6"/>
       <c r="B1661" s="7" t="s">
-        <v>2496</v>
+        <v>2498</v>
       </c>
       <c r="C1661" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1661" s="8">
-        <v>55</v>
+        <v>7</v>
       </c>
       <c r="E1661" s="8">
-        <v>28</v>
+        <v>875</v>
       </c>
       <c r="F1661" s="9">
         <f t="shared" si="26"/>
-        <v>1540</v>
+        <v>6125</v>
       </c>
       <c r="G1661" s="7" t="s">
         <v>2457</v>
@@ -68018,20 +68018,20 @@
     <row r="1662" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1662" s="6"/>
       <c r="B1662" s="7" t="s">
-        <v>2498</v>
+        <v>2499</v>
       </c>
       <c r="C1662" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1662" s="8">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="E1662" s="8">
-        <v>875</v>
+        <v>38</v>
       </c>
       <c r="F1662" s="9">
         <f t="shared" si="26"/>
-        <v>6125</v>
+        <v>570</v>
       </c>
       <c r="G1662" s="7" t="s">
         <v>2457</v>
@@ -68050,22 +68050,24 @@
       </c>
     </row>
     <row r="1663" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1663" s="6"/>
+      <c r="A1663" s="6" t="s">
+        <v>833</v>
+      </c>
       <c r="B1663" s="7" t="s">
-        <v>2499</v>
+        <v>834</v>
       </c>
       <c r="C1663" s="7" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="D1663" s="8">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="E1663" s="8">
-        <v>38</v>
+        <v>125</v>
       </c>
       <c r="F1663" s="9">
         <f t="shared" si="26"/>
-        <v>570</v>
+        <v>250</v>
       </c>
       <c r="G1663" s="7" t="s">
         <v>2457</v>
@@ -68084,24 +68086,24 @@
       </c>
     </row>
     <row r="1664" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1664" s="6" t="s">
-        <v>833</v>
+      <c r="A1664" s="30" t="s">
+        <v>2480</v>
       </c>
       <c r="B1664" s="7" t="s">
-        <v>834</v>
+        <v>2500</v>
       </c>
       <c r="C1664" s="7" t="s">
-        <v>46</v>
+        <v>713</v>
       </c>
       <c r="D1664" s="8">
-        <v>2</v>
+        <v>100</v>
       </c>
       <c r="E1664" s="8">
-        <v>125</v>
+        <v>58</v>
       </c>
       <c r="F1664" s="9">
         <f t="shared" si="26"/>
-        <v>250</v>
+        <v>5800</v>
       </c>
       <c r="G1664" s="7" t="s">
         <v>2457</v>
@@ -68121,23 +68123,23 @@
     </row>
     <row r="1665" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1665" s="30" t="s">
-        <v>2480</v>
+        <v>2494</v>
       </c>
       <c r="B1665" s="7" t="s">
-        <v>2500</v>
+        <v>2501</v>
       </c>
       <c r="C1665" s="7" t="s">
-        <v>713</v>
+        <v>21</v>
       </c>
       <c r="D1665" s="8">
-        <v>100</v>
+        <v>6</v>
       </c>
       <c r="E1665" s="8">
-        <v>58</v>
+        <v>25</v>
       </c>
       <c r="F1665" s="9">
         <f t="shared" si="26"/>
-        <v>5800</v>
+        <v>150</v>
       </c>
       <c r="G1665" s="7" t="s">
         <v>2457</v>
@@ -68157,23 +68159,23 @@
     </row>
     <row r="1666" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1666" s="30" t="s">
-        <v>2494</v>
+        <v>2502</v>
       </c>
       <c r="B1666" s="7" t="s">
-        <v>2501</v>
+        <v>840</v>
       </c>
       <c r="C1666" s="7" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="D1666" s="8">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E1666" s="8">
-        <v>25</v>
+        <v>95</v>
       </c>
       <c r="F1666" s="9">
         <f t="shared" si="26"/>
-        <v>150</v>
+        <v>1140</v>
       </c>
       <c r="G1666" s="7" t="s">
         <v>2457</v>
@@ -68193,23 +68195,23 @@
     </row>
     <row r="1667" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1667" s="30" t="s">
-        <v>2502</v>
+        <v>2503</v>
       </c>
       <c r="B1667" s="7" t="s">
-        <v>840</v>
+        <v>2504</v>
       </c>
       <c r="C1667" s="7" t="s">
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="D1667" s="8">
         <v>12</v>
       </c>
       <c r="E1667" s="8">
-        <v>95</v>
+        <v>55</v>
       </c>
       <c r="F1667" s="9">
         <f t="shared" si="26"/>
-        <v>1140</v>
+        <v>660</v>
       </c>
       <c r="G1667" s="7" t="s">
         <v>2457</v>
@@ -68229,23 +68231,23 @@
     </row>
     <row r="1668" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1668" s="30" t="s">
-        <v>2503</v>
+        <v>2505</v>
       </c>
       <c r="B1668" s="7" t="s">
-        <v>2504</v>
+        <v>2083</v>
       </c>
       <c r="C1668" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1668" s="8">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E1668" s="8">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="F1668" s="9">
         <f t="shared" si="26"/>
-        <v>660</v>
+        <v>768</v>
       </c>
       <c r="G1668" s="7" t="s">
         <v>2457</v>
@@ -68265,23 +68267,23 @@
     </row>
     <row r="1669" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1669" s="30" t="s">
-        <v>2505</v>
+        <v>2506</v>
       </c>
       <c r="B1669" s="7" t="s">
-        <v>2083</v>
+        <v>2507</v>
       </c>
       <c r="C1669" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1669" s="8">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="E1669" s="8">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="F1669" s="9">
         <f t="shared" si="26"/>
-        <v>768</v>
+        <v>330</v>
       </c>
       <c r="G1669" s="7" t="s">
         <v>2457</v>
@@ -68301,23 +68303,23 @@
     </row>
     <row r="1670" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1670" s="30" t="s">
-        <v>2506</v>
+        <v>2508</v>
       </c>
       <c r="B1670" s="7" t="s">
-        <v>2507</v>
+        <v>2509</v>
       </c>
       <c r="C1670" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1670" s="8">
-        <v>6</v>
+        <v>60</v>
       </c>
       <c r="E1670" s="8">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="F1670" s="9">
         <f t="shared" si="26"/>
-        <v>330</v>
+        <v>1500</v>
       </c>
       <c r="G1670" s="7" t="s">
         <v>2457</v>
@@ -68337,10 +68339,10 @@
     </row>
     <row r="1671" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1671" s="30" t="s">
-        <v>2508</v>
+        <v>2510</v>
       </c>
       <c r="B1671" s="7" t="s">
-        <v>2509</v>
+        <v>2511</v>
       </c>
       <c r="C1671" s="7" t="s">
         <v>21</v>
@@ -68349,11 +68351,11 @@
         <v>60</v>
       </c>
       <c r="E1671" s="8">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F1671" s="9">
         <f t="shared" si="26"/>
-        <v>1500</v>
+        <v>1200</v>
       </c>
       <c r="G1671" s="7" t="s">
         <v>2457</v>
@@ -68365,7 +68367,7 @@
         <v>534</v>
       </c>
       <c r="J1671" s="7" t="s">
-        <v>2497</v>
+        <v>2512</v>
       </c>
       <c r="K1671" s="10" t="s">
         <v>1793</v>
@@ -68373,23 +68375,23 @@
     </row>
     <row r="1672" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1672" s="30" t="s">
-        <v>2510</v>
+        <v>2513</v>
       </c>
       <c r="B1672" s="7" t="s">
-        <v>2511</v>
+        <v>2514</v>
       </c>
       <c r="C1672" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1672" s="8">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="E1672" s="8">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F1672" s="9">
         <f t="shared" si="26"/>
-        <v>1200</v>
+        <v>500</v>
       </c>
       <c r="G1672" s="7" t="s">
         <v>2457</v>
@@ -68409,23 +68411,23 @@
     </row>
     <row r="1673" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1673" s="30" t="s">
-        <v>2513</v>
+        <v>2515</v>
       </c>
       <c r="B1673" s="7" t="s">
-        <v>2514</v>
+        <v>2516</v>
       </c>
       <c r="C1673" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1673" s="8">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="E1673" s="8">
-        <v>25</v>
+        <v>75</v>
       </c>
       <c r="F1673" s="9">
         <f t="shared" si="26"/>
-        <v>500</v>
+        <v>75</v>
       </c>
       <c r="G1673" s="7" t="s">
         <v>2457</v>
@@ -68445,10 +68447,10 @@
     </row>
     <row r="1674" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1674" s="30" t="s">
-        <v>2515</v>
+        <v>2517</v>
       </c>
       <c r="B1674" s="7" t="s">
-        <v>2516</v>
+        <v>2518</v>
       </c>
       <c r="C1674" s="7" t="s">
         <v>21</v>
@@ -68457,11 +68459,11 @@
         <v>1</v>
       </c>
       <c r="E1674" s="8">
-        <v>75</v>
+        <v>35</v>
       </c>
       <c r="F1674" s="9">
         <f t="shared" si="26"/>
-        <v>75</v>
+        <v>35</v>
       </c>
       <c r="G1674" s="7" t="s">
         <v>2457</v>
@@ -68481,23 +68483,23 @@
     </row>
     <row r="1675" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1675" s="30" t="s">
-        <v>2517</v>
+        <v>2519</v>
       </c>
       <c r="B1675" s="7" t="s">
-        <v>2518</v>
+        <v>2520</v>
       </c>
       <c r="C1675" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1675" s="8">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E1675" s="8">
-        <v>35</v>
+        <v>75</v>
       </c>
       <c r="F1675" s="9">
         <f t="shared" si="26"/>
-        <v>35</v>
+        <v>300</v>
       </c>
       <c r="G1675" s="7" t="s">
         <v>2457</v>
@@ -68517,71 +68519,71 @@
     </row>
     <row r="1676" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1676" s="30" t="s">
-        <v>2519</v>
+        <v>216</v>
       </c>
       <c r="B1676" s="7" t="s">
-        <v>2520</v>
+        <v>2521</v>
       </c>
       <c r="C1676" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1676" s="8">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E1676" s="8">
-        <v>75</v>
+        <v>200</v>
       </c>
       <c r="F1676" s="9">
         <f t="shared" si="26"/>
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="G1676" s="7" t="s">
-        <v>2457</v>
+        <v>2522</v>
       </c>
       <c r="H1676" s="10" t="s">
-        <v>1789</v>
+        <v>2523</v>
       </c>
       <c r="I1676" s="7" t="s">
-        <v>534</v>
+        <v>129</v>
       </c>
       <c r="J1676" s="7" t="s">
-        <v>2512</v>
+        <v>2524</v>
       </c>
       <c r="K1676" s="10" t="s">
-        <v>1793</v>
+        <v>2525</v>
       </c>
     </row>
     <row r="1677" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1677" s="30" t="s">
-        <v>216</v>
+        <v>806</v>
       </c>
       <c r="B1677" s="7" t="s">
-        <v>2521</v>
+        <v>2526</v>
       </c>
       <c r="C1677" s="7" t="s">
-        <v>21</v>
+        <v>62</v>
       </c>
       <c r="D1677" s="8">
-        <v>2</v>
+        <v>266</v>
       </c>
       <c r="E1677" s="8">
-        <v>200</v>
+        <v>85</v>
       </c>
       <c r="F1677" s="9">
         <f t="shared" si="26"/>
-        <v>400</v>
+        <v>22610</v>
       </c>
       <c r="G1677" s="7" t="s">
-        <v>2522</v>
+        <v>2527</v>
       </c>
       <c r="H1677" s="10" t="s">
         <v>2523</v>
       </c>
       <c r="I1677" s="7" t="s">
-        <v>129</v>
+        <v>77</v>
       </c>
       <c r="J1677" s="7" t="s">
-        <v>2524</v>
+        <v>2528</v>
       </c>
       <c r="K1677" s="10" t="s">
         <v>2525</v>
@@ -68589,23 +68591,23 @@
     </row>
     <row r="1678" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1678" s="30" t="s">
-        <v>806</v>
+        <v>2529</v>
       </c>
       <c r="B1678" s="7" t="s">
-        <v>2526</v>
+        <v>2530</v>
       </c>
       <c r="C1678" s="7" t="s">
         <v>62</v>
       </c>
       <c r="D1678" s="8">
-        <v>266</v>
+        <v>568</v>
       </c>
       <c r="E1678" s="8">
-        <v>85</v>
+        <v>25</v>
       </c>
       <c r="F1678" s="9">
         <f t="shared" si="26"/>
-        <v>22610</v>
+        <v>14200</v>
       </c>
       <c r="G1678" s="7" t="s">
         <v>2527</v>
@@ -68625,35 +68627,35 @@
     </row>
     <row r="1679" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1679" s="30" t="s">
-        <v>2529</v>
+        <v>2531</v>
       </c>
       <c r="B1679" s="7" t="s">
-        <v>2530</v>
+        <v>2532</v>
       </c>
       <c r="C1679" s="7" t="s">
-        <v>62</v>
+        <v>21</v>
       </c>
       <c r="D1679" s="8">
-        <v>568</v>
+        <v>5</v>
       </c>
       <c r="E1679" s="8">
-        <v>25</v>
+        <v>4000</v>
       </c>
       <c r="F1679" s="9">
         <f t="shared" si="26"/>
-        <v>14200</v>
+        <v>20000</v>
       </c>
       <c r="G1679" s="7" t="s">
-        <v>2527</v>
+        <v>2533</v>
       </c>
       <c r="H1679" s="10" t="s">
-        <v>2523</v>
+        <v>2534</v>
       </c>
       <c r="I1679" s="7" t="s">
-        <v>77</v>
+        <v>57</v>
       </c>
       <c r="J1679" s="7" t="s">
-        <v>2528</v>
+        <v>2535</v>
       </c>
       <c r="K1679" s="10" t="s">
         <v>2525</v>
@@ -68661,23 +68663,23 @@
     </row>
     <row r="1680" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1680" s="30" t="s">
-        <v>2531</v>
+        <v>577</v>
       </c>
       <c r="B1680" s="7" t="s">
-        <v>2532</v>
+        <v>2536</v>
       </c>
       <c r="C1680" s="7" t="s">
-        <v>21</v>
+        <v>62</v>
       </c>
       <c r="D1680" s="8">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="E1680" s="8">
-        <v>4000</v>
+        <v>263.14999999999998</v>
       </c>
       <c r="F1680" s="9">
         <f t="shared" si="26"/>
-        <v>20000</v>
+        <v>8420.7999999999993</v>
       </c>
       <c r="G1680" s="7" t="s">
         <v>2533</v>
@@ -68697,23 +68699,23 @@
     </row>
     <row r="1681" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1681" s="30" t="s">
-        <v>577</v>
+        <v>699</v>
       </c>
       <c r="B1681" s="7" t="s">
-        <v>2536</v>
+        <v>2537</v>
       </c>
       <c r="C1681" s="7" t="s">
         <v>62</v>
       </c>
       <c r="D1681" s="8">
-        <v>32</v>
+        <v>60</v>
       </c>
       <c r="E1681" s="8">
         <v>263.14999999999998</v>
       </c>
       <c r="F1681" s="9">
         <f t="shared" si="26"/>
-        <v>8420.7999999999993</v>
+        <v>15788.999999999998</v>
       </c>
       <c r="G1681" s="7" t="s">
         <v>2533</v>
@@ -68733,59 +68735,59 @@
     </row>
     <row r="1682" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1682" s="30" t="s">
-        <v>699</v>
-      </c>
-      <c r="B1682" s="7" t="s">
-        <v>2537</v>
+        <v>157</v>
+      </c>
+      <c r="B1682" s="10" t="s">
+        <v>2538</v>
       </c>
       <c r="C1682" s="7" t="s">
-        <v>62</v>
+        <v>21</v>
       </c>
       <c r="D1682" s="8">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="E1682" s="8">
-        <v>263.14999999999998</v>
+        <v>555.75</v>
       </c>
       <c r="F1682" s="9">
-        <f t="shared" si="26"/>
-        <v>15788.999999999998</v>
+        <f>E1682*D1682</f>
+        <v>5557.5</v>
       </c>
       <c r="G1682" s="7" t="s">
-        <v>2533</v>
+        <v>2539</v>
       </c>
       <c r="H1682" s="10" t="s">
-        <v>2534</v>
+        <v>2332</v>
       </c>
       <c r="I1682" s="7" t="s">
-        <v>57</v>
+        <v>144</v>
       </c>
       <c r="J1682" s="7" t="s">
-        <v>2535</v>
-      </c>
-      <c r="K1682" s="10" t="s">
-        <v>2525</v>
+        <v>2540</v>
+      </c>
+      <c r="K1682" s="10">
+        <v>46363</v>
       </c>
     </row>
     <row r="1683" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1683" s="30" t="s">
-        <v>157</v>
+        <v>2541</v>
       </c>
       <c r="B1683" s="10" t="s">
-        <v>2538</v>
+        <v>2542</v>
       </c>
       <c r="C1683" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1683" s="8">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E1683" s="8">
-        <v>555.75</v>
+        <v>1054</v>
       </c>
       <c r="F1683" s="9">
-        <f>E1683*D1683</f>
-        <v>5557.5</v>
+        <f t="shared" ref="F1683:F1692" si="27">E1683*D1683</f>
+        <v>1054</v>
       </c>
       <c r="G1683" s="7" t="s">
         <v>2539</v>
@@ -68805,10 +68807,10 @@
     </row>
     <row r="1684" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1684" s="30" t="s">
-        <v>2541</v>
+        <v>2543</v>
       </c>
       <c r="B1684" s="10" t="s">
-        <v>2542</v>
+        <v>2544</v>
       </c>
       <c r="C1684" s="7" t="s">
         <v>21</v>
@@ -68817,11 +68819,11 @@
         <v>1</v>
       </c>
       <c r="E1684" s="8">
-        <v>1054</v>
+        <v>1266.99</v>
       </c>
       <c r="F1684" s="9">
-        <f t="shared" ref="F1684:F1693" si="27">E1684*D1684</f>
-        <v>1054</v>
+        <f t="shared" si="27"/>
+        <v>1266.99</v>
       </c>
       <c r="G1684" s="7" t="s">
         <v>2539</v>
@@ -68841,23 +68843,23 @@
     </row>
     <row r="1685" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1685" s="30" t="s">
-        <v>2543</v>
+        <v>2545</v>
       </c>
       <c r="B1685" s="10" t="s">
-        <v>2544</v>
+        <v>2546</v>
       </c>
       <c r="C1685" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1685" s="8">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E1685" s="8">
-        <v>1266.99</v>
+        <v>1160.5</v>
       </c>
       <c r="F1685" s="9">
         <f t="shared" si="27"/>
-        <v>1266.99</v>
+        <v>9284</v>
       </c>
       <c r="G1685" s="7" t="s">
         <v>2539</v>
@@ -68877,23 +68879,23 @@
     </row>
     <row r="1686" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1686" s="30" t="s">
-        <v>2545</v>
+        <v>2547</v>
       </c>
       <c r="B1686" s="10" t="s">
-        <v>2546</v>
+        <v>2548</v>
       </c>
       <c r="C1686" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1686" s="8">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E1686" s="8">
-        <v>1160.5</v>
+        <v>292.5</v>
       </c>
       <c r="F1686" s="9">
-        <f t="shared" si="27"/>
-        <v>9284</v>
+        <f>E1686*D1686</f>
+        <v>292.5</v>
       </c>
       <c r="G1686" s="7" t="s">
         <v>2539</v>
@@ -68913,10 +68915,10 @@
     </row>
     <row r="1687" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1687" s="30" t="s">
-        <v>2547</v>
+        <v>2549</v>
       </c>
       <c r="B1687" s="10" t="s">
-        <v>2548</v>
+        <v>2550</v>
       </c>
       <c r="C1687" s="7" t="s">
         <v>21</v>
@@ -68925,11 +68927,11 @@
         <v>1</v>
       </c>
       <c r="E1687" s="8">
-        <v>292.5</v>
+        <v>1930.5</v>
       </c>
       <c r="F1687" s="9">
-        <f>E1687*D1687</f>
-        <v>292.5</v>
+        <f t="shared" si="27"/>
+        <v>1930.5</v>
       </c>
       <c r="G1687" s="7" t="s">
         <v>2539</v>
@@ -68949,23 +68951,23 @@
     </row>
     <row r="1688" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1688" s="30" t="s">
-        <v>2549</v>
+        <v>904</v>
       </c>
       <c r="B1688" s="10" t="s">
-        <v>2550</v>
+        <v>2551</v>
       </c>
       <c r="C1688" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1688" s="8">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="E1688" s="8">
-        <v>1930.5</v>
+        <v>204.75</v>
       </c>
       <c r="F1688" s="9">
         <f t="shared" si="27"/>
-        <v>1930.5</v>
+        <v>3071.25</v>
       </c>
       <c r="G1688" s="7" t="s">
         <v>2539</v>
@@ -68985,23 +68987,23 @@
     </row>
     <row r="1689" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1689" s="30" t="s">
-        <v>904</v>
+        <v>2552</v>
       </c>
       <c r="B1689" s="10" t="s">
-        <v>2551</v>
+        <v>2553</v>
       </c>
       <c r="C1689" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D1689" s="8">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="E1689" s="8">
-        <v>204.75</v>
+        <v>175.5</v>
       </c>
       <c r="F1689" s="9">
         <f t="shared" si="27"/>
-        <v>3071.25</v>
+        <v>175.5</v>
       </c>
       <c r="G1689" s="7" t="s">
         <v>2539</v>
@@ -69021,35 +69023,35 @@
     </row>
     <row r="1690" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1690" s="30" t="s">
-        <v>2552</v>
+        <v>201</v>
       </c>
       <c r="B1690" s="10" t="s">
-        <v>2553</v>
-      </c>
-      <c r="C1690" s="7" t="s">
+        <v>2554</v>
+      </c>
+      <c r="C1690" s="10" t="s">
         <v>21</v>
       </c>
       <c r="D1690" s="8">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E1690" s="8">
-        <v>175.5</v>
+        <v>550</v>
       </c>
       <c r="F1690" s="9">
         <f t="shared" si="27"/>
-        <v>175.5</v>
+        <v>2750</v>
       </c>
       <c r="G1690" s="7" t="s">
-        <v>2539</v>
+        <v>2555</v>
       </c>
       <c r="H1690" s="10" t="s">
-        <v>2332</v>
+        <v>2556</v>
       </c>
       <c r="I1690" s="7" t="s">
-        <v>144</v>
-      </c>
-      <c r="J1690" s="7" t="s">
-        <v>2540</v>
+        <v>203</v>
+      </c>
+      <c r="J1690" s="10" t="s">
+        <v>2557</v>
       </c>
       <c r="K1690" s="10">
         <v>46363</v>
@@ -69057,23 +69059,23 @@
     </row>
     <row r="1691" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1691" s="30" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="B1691" s="10" t="s">
-        <v>2554</v>
+        <v>2558</v>
       </c>
       <c r="C1691" s="10" t="s">
         <v>21</v>
       </c>
       <c r="D1691" s="8">
-        <v>5</v>
+        <v>50</v>
       </c>
       <c r="E1691" s="8">
-        <v>550</v>
+        <v>15</v>
       </c>
       <c r="F1691" s="9">
         <f t="shared" si="27"/>
-        <v>2750</v>
+        <v>750</v>
       </c>
       <c r="G1691" s="7" t="s">
         <v>2555</v>
@@ -69093,23 +69095,23 @@
     </row>
     <row r="1692" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1692" s="30" t="s">
-        <v>205</v>
+        <v>297</v>
       </c>
       <c r="B1692" s="10" t="s">
-        <v>2558</v>
+        <v>2559</v>
       </c>
       <c r="C1692" s="10" t="s">
         <v>21</v>
       </c>
       <c r="D1692" s="8">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="E1692" s="8">
-        <v>15</v>
+        <v>800</v>
       </c>
       <c r="F1692" s="9">
         <f t="shared" si="27"/>
-        <v>750</v>
+        <v>3200</v>
       </c>
       <c r="G1692" s="7" t="s">
         <v>2555</v>
@@ -69129,59 +69131,59 @@
     </row>
     <row r="1693" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1693" s="30" t="s">
-        <v>297</v>
-      </c>
-      <c r="B1693" s="10" t="s">
-        <v>2559</v>
+        <v>1528</v>
+      </c>
+      <c r="B1693" s="7" t="s">
+        <v>2560</v>
       </c>
       <c r="C1693" s="10" t="s">
         <v>21</v>
       </c>
       <c r="D1693" s="8">
-        <v>4</v>
+        <v>79</v>
       </c>
       <c r="E1693" s="8">
-        <v>800</v>
+        <v>1666</v>
       </c>
       <c r="F1693" s="9">
-        <f t="shared" si="27"/>
-        <v>3200</v>
+        <f t="shared" si="26"/>
+        <v>131614</v>
       </c>
       <c r="G1693" s="7" t="s">
-        <v>2555</v>
+        <v>2561</v>
       </c>
       <c r="H1693" s="10" t="s">
         <v>2556</v>
       </c>
       <c r="I1693" s="7" t="s">
-        <v>203</v>
-      </c>
-      <c r="J1693" s="10" t="s">
-        <v>2557</v>
-      </c>
-      <c r="K1693" s="10">
-        <v>46363</v>
+        <v>2562</v>
+      </c>
+      <c r="J1693" s="7" t="s">
+        <v>2563</v>
+      </c>
+      <c r="K1693" s="10" t="s">
+        <v>2564</v>
       </c>
     </row>
     <row r="1694" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1694" s="30" t="s">
-        <v>1528</v>
+        <v>2565</v>
       </c>
       <c r="B1694" s="7" t="s">
-        <v>2560</v>
+        <v>2566</v>
       </c>
       <c r="C1694" s="10" t="s">
         <v>21</v>
       </c>
       <c r="D1694" s="8">
-        <v>79</v>
+        <v>121</v>
       </c>
       <c r="E1694" s="8">
-        <v>1666</v>
+        <v>1842</v>
       </c>
       <c r="F1694" s="9">
         <f t="shared" si="26"/>
-        <v>131614</v>
+        <v>222882</v>
       </c>
       <c r="G1694" s="7" t="s">
         <v>2561</v>
@@ -69200,60 +69202,60 @@
       </c>
     </row>
     <row r="1695" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1695" s="30" t="s">
-        <v>2565</v>
+      <c r="A1695" s="6" t="s">
+        <v>2567</v>
       </c>
       <c r="B1695" s="7" t="s">
-        <v>2566</v>
+        <v>2568</v>
       </c>
       <c r="C1695" s="10" t="s">
         <v>21</v>
       </c>
       <c r="D1695" s="8">
-        <v>121</v>
+        <v>18</v>
       </c>
       <c r="E1695" s="8">
-        <v>1842</v>
+        <v>871.35</v>
       </c>
       <c r="F1695" s="9">
         <f t="shared" si="26"/>
-        <v>222882</v>
+        <v>15684.300000000001</v>
       </c>
       <c r="G1695" s="7" t="s">
-        <v>2561</v>
-      </c>
-      <c r="H1695" s="10" t="s">
-        <v>2556</v>
+        <v>2569</v>
+      </c>
+      <c r="H1695" s="10">
+        <v>46327</v>
       </c>
       <c r="I1695" s="7" t="s">
-        <v>2562</v>
+        <v>804</v>
       </c>
       <c r="J1695" s="7" t="s">
-        <v>2563</v>
+        <v>2570</v>
       </c>
       <c r="K1695" s="10" t="s">
-        <v>2564</v>
+        <v>71</v>
       </c>
     </row>
     <row r="1696" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1696" s="6" t="s">
-        <v>2567</v>
+        <v>2571</v>
       </c>
       <c r="B1696" s="7" t="s">
-        <v>2568</v>
+        <v>2572</v>
       </c>
       <c r="C1696" s="10" t="s">
         <v>21</v>
       </c>
       <c r="D1696" s="8">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E1696" s="8">
-        <v>871.35</v>
+        <v>261.41000000000003</v>
       </c>
       <c r="F1696" s="9">
         <f t="shared" si="26"/>
-        <v>15684.300000000001</v>
+        <v>4966.7900000000009</v>
       </c>
       <c r="G1696" s="7" t="s">
         <v>2569</v>
@@ -69272,11 +69274,9 @@
       </c>
     </row>
     <row r="1697" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1697" s="6" t="s">
-        <v>2571</v>
-      </c>
+      <c r="A1697" s="6"/>
       <c r="B1697" s="7" t="s">
-        <v>2572</v>
+        <v>2573</v>
       </c>
       <c r="C1697" s="10" t="s">
         <v>21</v>
@@ -69284,12 +69284,12 @@
       <c r="D1697" s="8">
         <v>19</v>
       </c>
-      <c r="E1697" s="8">
-        <v>261.41000000000003</v>
+      <c r="E1697" s="19">
+        <v>529.20000000000005</v>
       </c>
       <c r="F1697" s="9">
         <f t="shared" si="26"/>
-        <v>4966.7900000000009</v>
+        <v>10054.800000000001</v>
       </c>
       <c r="G1697" s="7" t="s">
         <v>2569</v>
@@ -69310,7 +69310,7 @@
     <row r="1698" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1698" s="6"/>
       <c r="B1698" s="7" t="s">
-        <v>2573</v>
+        <v>2574</v>
       </c>
       <c r="C1698" s="10" t="s">
         <v>21</v>
@@ -69318,12 +69318,12 @@
       <c r="D1698" s="8">
         <v>19</v>
       </c>
-      <c r="E1698" s="19">
-        <v>529.20000000000005</v>
+      <c r="E1698" s="8">
+        <v>120</v>
       </c>
       <c r="F1698" s="9">
         <f t="shared" si="26"/>
-        <v>10054.800000000001</v>
+        <v>2280</v>
       </c>
       <c r="G1698" s="7" t="s">
         <v>2569</v>
@@ -69341,53 +69341,19 @@
         <v>71</v>
       </c>
     </row>
-    <row r="1699" spans="1:11" s="12" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1699" s="6"/>
-      <c r="B1699" s="7" t="s">
-        <v>2574</v>
-      </c>
-      <c r="C1699" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="D1699" s="8">
-        <v>19</v>
-      </c>
-      <c r="E1699" s="8">
-        <v>120</v>
-      </c>
-      <c r="F1699" s="9">
-        <f t="shared" si="26"/>
-        <v>2280</v>
-      </c>
-      <c r="G1699" s="7" t="s">
-        <v>2569</v>
-      </c>
-      <c r="H1699" s="10">
-        <v>46327</v>
-      </c>
-      <c r="I1699" s="7" t="s">
-        <v>804</v>
-      </c>
-      <c r="J1699" s="7" t="s">
-        <v>2570</v>
-      </c>
-      <c r="K1699" s="10" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="1700" spans="1:11" ht="22.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="C1700" s="20"/>
-      <c r="D1700" s="21"/>
-      <c r="E1700" s="21"/>
-      <c r="F1700" s="33">
-        <f>SUM(F2:F1699)</f>
-        <v>27668891.124196012</v>
-      </c>
-      <c r="G1700" s="20"/>
-      <c r="H1700" s="22"/>
-      <c r="I1700" s="20"/>
-      <c r="J1700" s="20"/>
-      <c r="K1700" s="22"/>
+    <row r="1699" spans="1:11" ht="22.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="C1699" s="20"/>
+      <c r="D1699" s="21"/>
+      <c r="E1699" s="21"/>
+      <c r="F1699" s="33">
+        <f>SUM(F2:F1698)</f>
+        <v>27668441.124196012</v>
+      </c>
+      <c r="G1699" s="20"/>
+      <c r="H1699" s="22"/>
+      <c r="I1699" s="20"/>
+      <c r="J1699" s="20"/>
+      <c r="K1699" s="22"/>
     </row>
   </sheetData>
   <phoneticPr fontId="10" type="noConversion"/>

</xml_diff>